<commit_message>
enhanced version of ATS,two logs file:one for just raw texts another for segmented sections
</commit_message>
<xml_diff>
--- a/output/all_candidates_ranked.xlsx
+++ b/output/all_candidates_ranked.xlsx
@@ -503,46 +503,46 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13-ResumeMominKhan 4y.pdf</t>
+          <t>25-Resumezeeshanzahoor3y+.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Momin Hyat Khan</t>
+          <t>Zeeshan Zahoor</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>mominhyatkhandeveloper@gmail.com</t>
+          <t>zeeshanzahoor409@gmail.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>03345674415</t>
+          <t>+923421905266</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://linkedin.com/in/mominhyatkhan</t>
+          <t>https://www.linkedin.com/in/zeeshan-zahoor-220b0b130</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://github.com/mominhyatkhan</t>
+          <t>https://github.com/zeeshanshaanu</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>material ui, github, javascript, next.js, git, eslint, typescript, prettier, axios, html, react query, tailwind css, redux, css, react</t>
+          <t>next.js, github, css, figma, lighthouse, javascript, typescript, git, responsive design, material ui, tailwind css, redux, redux toolkit, react.js, bootstrap, vercel, websockets, react, netlify</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>4 years 0 months</t>
+          <t>3 years 0 months</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -551,7 +551,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Bachelor / No major degree found but there is a university mention</t>
+          <t>🎓 BS in Computer Science (2016 – 2020) | Gov’t Post Graduate College, Haripur</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -569,42 +569,46 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>28-zeeshaan updated4y+.pdf</t>
+          <t>13-ResumeMominKhan 4y.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Zeeshan Zahoor</t>
+          <t>Momin Hyat Khan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>zeeshanzahoor409@gmail.com</t>
+          <t>mominhyatkhandeveloper@gmail.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>+923421905266</t>
+          <t>03345674415</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/zeeshan-zahoor-220b0b130</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://linkedin.com/in/mominhyatkhan</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://github.com/mominhyatkhan</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>material ui, github, redux, netlify, vercel, javascript, responsive design, redux toolkit, typescript, bootstrap, websockets, css, lighthouse, next.js, react, git, react.js, tailwind css, figma</t>
+          <t>axios, javascript, next.js, material ui, html, github, typescript, git, tailwind css, redux, react, css, react query, eslint, prettier</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>3 years 0 months</t>
+          <t>4 years 0 months</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -613,7 +617,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>🎓 BS in Computer Science (2016 – 2020) | Gov’t Post Graduate College, Haripur</t>
+          <t>Bachelor / No major degree found but there is a university mention</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -622,7 +626,7 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>85.69</v>
+        <v>87.69</v>
       </c>
       <c r="N3" t="n">
         <v>2</v>
@@ -631,7 +635,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>25-Resumezeeshanzahoor3y+.pdf</t>
+          <t>28-zeeshaan updated4y+.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -654,10 +658,14 @@
           <t>https://www.linkedin.com/in/zeeshan-zahoor-220b0b130</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://github.com/zeeshanshaanu</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>material ui, github, redux, netlify, vercel, javascript, responsive design, redux toolkit, typescript, bootstrap, websockets, css, lighthouse, next.js, react, git, react.js, tailwind css, figma</t>
+          <t>next.js, github, css, figma, lighthouse, javascript, typescript, git, responsive design, material ui, tailwind css, redux, redux toolkit, react.js, bootstrap, vercel, websockets, react, netlify</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -684,7 +692,7 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>85.69</v>
+        <v>87.69</v>
       </c>
       <c r="N4" t="n">
         <v>3</v>
@@ -723,7 +731,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>github, redux, netlify, vercel, seo optimization, cypress, javascript, responsive design, typescript, jest, progressive web apps, css, babel, next.js, webpack, single page applications, vue.js, lazy loading, react, state management, git, react.js, styled components, react testing library, github actions, code splitting, tailwind css, graphql, figma</t>
+          <t>next.js, github, jest, vue.js, lazy loading, css, cypress, state management, figma, javascript, graphql, typescript, git, code splitting, progressive web apps, single page applications, react testing library, responsive design, styled components, tailwind css, redux, webpack, react.js, vercel, seo optimization, react, netlify, babel, github actions</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -784,12 +792,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>http://github.com/ayazcoder</t>
+          <t>https://github.com/ayazcoder</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>material ui, github, javascript, git, react.js, github actions, tailwind css, react, css, react hooks</t>
+          <t>javascript, material ui, github, git, tailwind css, react hooks, react, css, github actions, react.js</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -851,7 +859,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>material ui, javascript, git, react.js, html, tailwind css, redux, css, react, figma, state management</t>
+          <t>javascript, material ui, html, git, tailwind css, redux, react, css, state management, figma, react.js</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -909,7 +917,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>material ui, github, javascript, next.js, git, react.js, typescript, bootstrap, tailwind css, css, adobe xd, react, figma</t>
+          <t>bootstrap, javascript, next.js, material ui, adobe xd, typescript, github, git, tailwind css, react, css, figma, react.js</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -967,7 +975,7 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>vite, npm, github, javascript, chrome devtools, git, react.js, bootstrap, html, tailwind css, css, yarn, react, figma</t>
+          <t>bootstrap, chrome devtools, javascript, npm, yarn, vite, html, github, git, tailwind css, react, css, figma, react.js</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1025,7 +1033,7 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>javascript, github, react.js, html, redux, css, react, state management</t>
+          <t>javascript, html, github, redux, react, css, state management, react.js</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1091,7 +1099,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>jquery, javascript, github, git, react.js, bootstrap, html, vue.js, tailwind css, chakra ui, css, react</t>
+          <t>chakra ui, bootstrap, javascript, jquery, html, github, git, tailwind css, vue.js, react, css, react.js</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1149,7 +1157,7 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>material ui, javascript, next.js, responsive design, react.js, typescript, html, tailwind css, css, react</t>
+          <t>javascript, next.js, responsive design, material ui, html, typescript, tailwind css, react, css, react.js</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1215,7 +1223,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>github, javascript, next.js, git, vercel, react.js, redux toolkit, react query, vue.js, redux, tailwind css, css, react, figma</t>
+          <t>javascript, next.js, vercel, github, git, tailwind css, redux, vue.js, react, css, react query, redux toolkit, figma, react.js</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1273,7 +1281,7 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>javascript, github, git, bootstrap, bitbucket, rest api</t>
+          <t>bootstrap, javascript, github, git, bitbucket, rest api</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1331,7 +1339,7 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>javascript, github, git, bootstrap, bitbucket, rest api</t>
+          <t>bootstrap, javascript, github, git, bitbucket, rest api</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1393,7 +1401,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>less, typescript, html, rest api, react, css, graphql</t>
+          <t>graphql, html, typescript, less, rest api, react, css</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1429,38 +1437,46 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>24-ResumeTayyabHussainshah.pdf</t>
+          <t>7-Muhammad Yasin - Software Engineer.pdf</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tayyab Hussain Shah</t>
+          <t>Muhammad Yasin Software Engineer</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>tayabsajid5@gmail.com</t>
+          <t>yasinwaheed11@gmail.com</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>+923365298230</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+          <t>+923026770777</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/yasinwahid111</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://github.com/YasinWahid</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>vite, github, javascript, next.js, git, vercel, sass, react.js, typescript, tailwind css, redux, angular, css, react, figma</t>
+          <t>bootstrap, javascript, responsive design, angular, html, github, typescript, git, react, css, figma, react.js</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1 years 4 months</t>
+          <t>1 years 2 months</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1469,16 +1485,16 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Software Engineering</t>
+          <t>Hifah Technologies | Abbottabad Bachelor of Software Engineering</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
+          <t>date_range via fuzzy-month + month-name + year-only</t>
         </is>
       </c>
       <c r="M17" t="n">
-        <v>62.95</v>
+        <v>63.21</v>
       </c>
       <c r="N17" t="n">
         <v>16</v>
@@ -1487,52 +1503,56 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12-ResumeIjlalSHAH-2y.pdf</t>
+          <t>24-ResumeTayyabHussainshah.pdf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ijlal Shah</t>
+          <t>Tayyab Hussain Shah</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ijlalshahzr@gmail.com</t>
+          <t>tayabsajid5@gmail.com</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>+923181669799</t>
+          <t>+923365298230</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>material ui, jquery, javascript, git, react.js, context api, redux toolkit, typescript, angular, bootstrap, html, lazy loading, redux, react, css, react hooks, state management</t>
+          <t>javascript, sass, next.js, angular, vite, vercel, github, typescript, git, tailwind css, redux, react, css, figma, react.js</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2 years 0 months</t>
+          <t>1 years 4 months</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr"/>
+          <t>bachelor</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Bachelor of Science in Software Engineering</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
       <c r="M18" t="n">
-        <v>62.69</v>
+        <v>62.95</v>
       </c>
       <c r="N18" t="n">
         <v>17</v>
@@ -1541,64 +1561,52 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>22-ResumeSaadAhmad-1y.pdf</t>
+          <t>12-ResumeIjlalSHAH-2y.pdf</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Saad Ahmad</t>
+          <t>Ijlal Shah</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>saadahmad6830879@gmail.com</t>
+          <t>ijlalshahzr@gmail.com</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>923176830879</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/in/saadahmad879</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>https://github.com/SaADii09</t>
-        </is>
-      </c>
+          <t>+923181669799</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>javascript, github, git, react.js, html, tailwind css, redux, css, react, state management</t>
+          <t>bootstrap, jquery, javascript, material ui, angular, html, typescript, git, context api, react hooks, redux, react, lazy loading, css, redux toolkit, state management, react.js</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0 years 8 months</t>
+          <t>2 years 0 months</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>0.7</v>
+        <v>2</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>bachelor</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>BS Computer Science</t>
-        </is>
-      </c>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M19" t="n">
-        <v>61.28</v>
+        <v>62.69</v>
       </c>
       <c r="N19" t="n">
         <v>18</v>
@@ -1607,42 +1615,46 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>7-Muhammad Yasin - Software Engineer.pdf</t>
+          <t>22-ResumeSaadAhmad-1y.pdf</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Muhammad Yasin Software Engineer</t>
+          <t>Saad Ahmad</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>yasinwaheed11@gmail.com</t>
+          <t>saadahmad6830879@gmail.com</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>+923026770777</t>
+          <t>923176830879</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/yasinwahid111</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
+          <t>https://linkedin.com/in/saadahmad879</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://github.com/SaADii09</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>github, javascript, git, responsive design, react.js, typescript, bootstrap, html, angular, css, react, figma</t>
+          <t>javascript, html, github, git, tailwind css, redux, react, css, state management, react.js</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1 years 2 months</t>
+          <t>0 years 8 months</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1651,16 +1663,16 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Hifah Technologies | Abbottabad Bachelor of Software Engineering</t>
+          <t>BS Computer Science</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
       <c r="M20" t="n">
-        <v>61.21</v>
+        <v>61.28</v>
       </c>
       <c r="N20" t="n">
         <v>19</v>
@@ -1691,7 +1703,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>github, git, jenkins, bitbucket, rest api</t>
+          <t>jenkins, github, git, bitbucket, rest api</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1752,12 +1764,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>http://github.com/Fahad12405/</t>
+          <t>https://github.com/Fahad12405</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>vite, github, html, redux, javascript, redux toolkit, typescript, postcss, bootstrap, css, jquery, next.js, webpack, context api, axios, vue.js, react, state management, git, react.js, tailwind css</t>
+          <t>next.js, github, vue.js, css, postcss, state management, javascript, typescript, git, tailwind css, redux, redux toolkit, webpack, react.js, axios, bootstrap, jquery, vite, html, context api, react</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1814,12 +1826,12 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://github.com/</t>
+          <t>https://github.com/model</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>github, rest api</t>
+          <t>rest api, github</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1885,7 +1897,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>npm, github, javascript, next.js, git, react.js, redux toolkit, react router, html, redux, css, yarn, react, vercel</t>
+          <t>javascript, next.js, npm, yarn, html, github, vercel, git, redux, react, css, redux toolkit, react router, react.js</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1951,7 +1963,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>javascript, github, git, html, css</t>
+          <t>javascript, html, github, git, css</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2017,7 +2029,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>javascript, github, git, html, css</t>
+          <t>javascript, html, github, git, css</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2083,7 +2095,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>github, rest api</t>
+          <t>rest api, github</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2140,7 +2152,7 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://github.com/</t>
+          <t>https://github.com/PROFILE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2181,22 +2193,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>data-scientist-resume-sample-template.pdf</t>
+          <t>Tanjiro_Bhatia_Resume_09-08-2022-19-15-13.pdf</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Robin Doe</t>
+          <t>Tanjiro Bhatia</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>fobin.doe@example.com</t>
+          <t>Tanjiro.bhatia67@gmail.com</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>123451234567090</t>
+          <t>9923312341</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -2204,11 +2216,11 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>8 years 6 months</t>
+          <t>6 years 0 months</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -2217,12 +2229,12 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>ba Eng al) - AMT</t>
+          <t>Bachelor / No major degree found but there is a university mention</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>date_range via year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -2235,34 +2247,42 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Tanjiro_Bhatia_Resume_09-08-2022-19-15-13.pdf</t>
+          <t>21-ResumeRehmanZeb2y+.pdf</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Tanjiro Bhatia</t>
+          <t>Resumerehmanzeb2Y+</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tanjiro.bhatia67@gmail.com</t>
+          <t>rehmanzeb2k17@gmail.com</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>9923312341</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr"/>
+          <t>+923119449029</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/rehmanzeb</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>bootstrap, javascript, next.js, responsive design, git, tailwind css, react, css, react.js</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>6 years 0 months</t>
+          <t>0 years 9 months</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>6</v>
+        <v>0.8</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -2271,16 +2291,16 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Bachelor / No major degree found but there is a university mention</t>
+          <t>BS Computer Science</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via fuzzy-month + month-name + year-only + month-only + year</t>
         </is>
       </c>
       <c r="M30" t="n">
-        <v>55</v>
+        <v>53.96</v>
       </c>
       <c r="N30" t="n">
         <v>29</v>
@@ -2289,60 +2309,56 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>21-ResumeRehmanZeb2y+.pdf</t>
+          <t>17-ResumeMuhammadShayan3y.pdf</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Resumerehmanzeb2Y+</t>
+          <t>Muhammad Shayan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>rehmanzeb2k17@gmail.com</t>
+          <t>kshayan091@gmail.com</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>+923119449029</t>
+          <t>+923168104861</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/rehmanzeb</t>
+          <t>https://www.linkedin.com/in/shayan-khan20</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>javascript, next.js, git, responsive design, react.js, bootstrap, tailwind css, css, react</t>
+          <t>javascript, next.js, material ui, typescript, github, seo optimization, redux, react, figma</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>0 years 9 months</t>
+          <t>1 years 11 months</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>0.8</v>
+        <v>1.9</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>bachelor</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>BS Computer Science</t>
-        </is>
-      </c>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + month-only + year</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
       <c r="M31" t="n">
-        <v>53.96</v>
+        <v>52.55</v>
       </c>
       <c r="N31" t="n">
         <v>30</v>
@@ -2351,56 +2367,48 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>17-ResumeMuhammadShayan3y.pdf</t>
+          <t>data-scientist-resume-sample-template.pdf</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Muhammad Shayan</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>kshayan091@gmail.com</t>
-        </is>
-      </c>
+          <t>Robin Doe</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>+923168104861</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/shayan-khan20</t>
-        </is>
-      </c>
+          <t>123451234567090</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>material ui, github, seo optimization, next.js, javascript, typescript, redux, react, figma</t>
-        </is>
-      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1 years 11 months</t>
+          <t>8 years 6 months</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>1.9</v>
+        <v>8.5</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr"/>
+          <t>bachelor</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ba Eng al) - AMT</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
+          <t>date_range via year-only</t>
         </is>
       </c>
       <c r="M32" t="n">
-        <v>52.55</v>
+        <v>52</v>
       </c>
       <c r="N32" t="n">
         <v>31</v>
@@ -2431,7 +2439,7 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>css, html, javascript</t>
+          <t>html, javascript, css</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2497,7 +2505,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>material ui, github, api's integration, bootstrap, tailwind css, redux, css, react, vercel</t>
+          <t>bootstrap, material ui, vercel, github, api's integration, tailwind css, redux, react, css</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2556,10 +2564,14 @@
           <t>https://linkedin.com/in/muhammad-luqman-khan-051047267</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://github.com/Luqmanoffical</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>github, javascript, react.js, typescript, bootstrap, html, netlify, css, react, figma</t>
+          <t>bootstrap, javascript, html, github, typescript, react, netlify, css, figma, react.js</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2586,7 +2598,7 @@
         </is>
       </c>
       <c r="M35" t="n">
-        <v>46.46</v>
+        <v>48.46</v>
       </c>
       <c r="N35" t="n">
         <v>34</v>
@@ -2595,52 +2607,64 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Riya_Bhatiya_Resume_09-08-2022-19-26-53.pdf</t>
+          <t>5-JAWADRESUME.pdf</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Riya Bhatiya</t>
+          <t>Jawad Ali</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>riya.bhatia67@gmail.com</t>
+          <t>jawadalikhan359@gmail.com</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>9923312341</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
+          <t>03139908709</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jawadali1535</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://github.com/JawadAli1535</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>axios, jquery, javascript, sass, vercel, github, typescript, git, tailwind css, redux, react, css</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>2 years 0 months</t>
+          <t>0 years 5 months</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>2</v>
+        <v>0.4</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>high school</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Bachelor Of Technology in Computer Science Freelance Mentor Of Data Structure and Algorithms</t>
+          <t>Nodejs(intermediate)</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via fuzzy-month + month-name + year-only</t>
         </is>
       </c>
       <c r="M36" t="n">
-        <v>45</v>
+        <v>45.71</v>
       </c>
       <c r="N36" t="n">
         <v>35</v>
@@ -2649,64 +2673,52 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>resume_juanjosecarin.pdf</t>
+          <t>Riya_Bhatiya_Resume_09-08-2022-19-26-53.pdf</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Juan Jose Carin</t>
+          <t>Riya Bhatiya</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>juanjose.carin@gmail.com</t>
+          <t>riya.bhatia67@gmail.com</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>940416503364590</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/in/juanjosecarin</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>https://github.com/juanjocarin/W261-Machine-Learning-At-Scale/blob/master/Week07-MrJob/MIDS-W261-2015-HWK-Week07-CarinLlopSatpati-groupZ.ipynb</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>github, git</t>
-        </is>
-      </c>
+          <t>9923312341</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1 years 2 months</t>
+          <t>2 years 0 months</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>master</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Master of Information and Data Science</t>
+          <t>Bachelor Of Technology in Computer Science Freelance Mentor Of Data Structure and Algorithms</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M37" t="n">
-        <v>44.74</v>
+        <v>45</v>
       </c>
       <c r="N37" t="n">
         <v>36</v>
@@ -2715,51 +2727,55 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>5-JAWADRESUME.pdf</t>
+          <t>resume_juanjosecarin.pdf</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Jawad Ali</t>
+          <t>Juan Jose Carin</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>jawadalikhan359@gmail.com</t>
+          <t>juanjose.carin@gmail.com</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>03139908709</t>
+          <t>940416503364590</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jawadali1535</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
+          <t>https://linkedin.com/in/juanjosecarin</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://github.com/juanjocarin/W261-Machine-Learning-At-Scale/blob/master/Week07-MrJob/MIDS-W261-2015-HWK-Week07-CarinLlopSatpati-groupZ.ipynb</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>jquery, github, javascript, git, sass, typescript, axios, tailwind css, redux, css, react, vercel</t>
+          <t>github, git</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>0 years 5 months</t>
+          <t>1 years 2 months</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>high school</t>
+          <t>master</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Nodejs(intermediate)</t>
+          <t>Master of Information and Data Science</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -2768,7 +2784,7 @@
         </is>
       </c>
       <c r="M38" t="n">
-        <v>43.71</v>
+        <v>44.74</v>
       </c>
       <c r="N38" t="n">
         <v>37</v>
@@ -2839,56 +2855,60 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Nitish Kumar.pdf</t>
+          <t>26-Sameer Khan Cv3y.pdf</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Nitish Kumar</t>
+          <t>Sameer Khan</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>xyz@gmail.com</t>
+          <t>berlanjan123@gmail.com</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>9977141714</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>https://github.com/vishalsingh17</t>
-        </is>
-      </c>
+          <t>+923169769253</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sameer-khan-660966251</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>css, html, github, git</t>
+          <t>bootstrap, next.js, html, github, react, css</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1 years 0 months</t>
+          <t>0 years 0 months</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr"/>
+          <t>bachelor</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Degree Bs Computer Science</t>
+        </is>
+      </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>none via none</t>
         </is>
       </c>
       <c r="M40" t="n">
-        <v>36.23</v>
+        <v>37.23</v>
       </c>
       <c r="N40" t="n">
         <v>39</v>
@@ -2897,42 +2917,42 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>3-AJSwatiResume.pdf</t>
+          <t>Nitish Kumar.pdf</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Abdullah Javed</t>
+          <t>Nitish Kumar</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>abdullah.javed9438@gmail.com</t>
+          <t>xyz@gmail.com</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>+923499377144</t>
+          <t>9977141714</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://github.com/AbdullahKhanSwati</t>
+          <t>https://github.com/vishalsingh17</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>jquery, github, javascript, netlify, responsive design, react.js, tailwind css, lazy loading, redux, react, css, react hooks, state management</t>
+          <t>html, github, css, git</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>0 years 0 months</t>
+          <t>1 years 0 months</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -2942,11 +2962,11 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>none via none</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M41" t="n">
-        <v>35.46</v>
+        <v>36.23</v>
       </c>
       <c r="N41" t="n">
         <v>40</v>
@@ -2955,29 +2975,33 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>26-Sameer Khan Cv3y.pdf</t>
+          <t>3-AJSwatiResume.pdf</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Sameer Khan</t>
+          <t>Abdullah Javed</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>berlanjan123@gmail.com</t>
+          <t>abdullah.javed9438@gmail.com</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>+923169769253</t>
+          <t>+923499377144</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://github.com/AbdullahKhanSwati</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>github, next.js, bootstrap, html, css, react</t>
+          <t>jquery, javascript, responsive design, github, tailwind css, react hooks, redux, react, lazy loading, css, netlify, state management, react.js</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2990,21 +3014,17 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>bachelor</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Degree Bs Computer Science</t>
-        </is>
-      </c>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
           <t>none via none</t>
         </is>
       </c>
       <c r="M42" t="n">
-        <v>34.23</v>
+        <v>35.46</v>
       </c>
       <c r="N42" t="n">
         <v>41</v>
@@ -3035,7 +3055,7 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>gitlab, git</t>
+          <t>git, gitlab</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">

</xml_diff>

<commit_message>
enhanced experience and education extraction
</commit_message>
<xml_diff>
--- a/output/all_candidates_ranked.xlsx
+++ b/output/all_candidates_ranked.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>responsive design, lighthouse, redux, javascript, websockets, react, vercel, next.js, figma, github, tailwind css, git, typescript, material ui, css, netlify, react.js, redux toolkit, bootstrap</t>
+          <t>bootstrap, redux toolkit, react, material ui, javascript, git, next.js, css, websockets, netlify, redux, figma, github, tailwind css, responsive design, typescript, vercel, lighthouse, react.js</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>html, github, material ui, css, git, eslint, tailwind css, axios, next.js, redux, react query, javascript, prettier, typescript, react</t>
+          <t>github, javascript, prettier, eslint, tailwind css, git, next.js, html, axios, react query, react, typescript, redux, css, material ui</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Bachelor / No major degree found but there is a university mention</t>
+          <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>responsive design, lighthouse, redux, javascript, websockets, react, vercel, next.js, figma, github, tailwind css, git, typescript, material ui, css, netlify, react.js, redux toolkit, bootstrap</t>
+          <t>bootstrap, redux toolkit, react, material ui, javascript, git, next.js, css, websockets, netlify, redux, figma, github, tailwind css, responsive design, typescript, vercel, lighthouse, react.js</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>responsive design, graphql, redux, github actions, cypress, javascript, code splitting, react, vercel, single page applications, next.js, seo optimization, styled components, figma, react testing library, github, babel, state management, tailwind css, progressive web apps, lazy loading, vue.js, typescript, webpack, git, css, netlify, jest, react.js</t>
+          <t>progressive web apps, jest, state management, react, webpack, javascript, git, next.js, code splitting, css, netlify, graphql, github actions, single page applications, redux, react testing library, vue.js, figma, babel, github, tailwind css, responsive design, cypress, typescript, vercel, lazy loading, styled components, seo optimization, react.js</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>github, material ui, css, tailwind css, react.js, github actions, javascript, git, react, react hooks</t>
+          <t>github, javascript, tailwind css, git, react hooks, github actions, react, css, material ui, react.js</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -859,7 +859,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>html, material ui, css, state management, tailwind css, redux, react.js, figma, javascript, git, react</t>
+          <t>javascript, state management, tailwind css, git, html, react, redux, css, material ui, figma, react.js</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -917,7 +917,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>github, material ui, css, tailwind css, next.js, react.js, bootstrap, figma, javascript, adobe xd, git, typescript, react</t>
+          <t>github, javascript, tailwind css, git, bootstrap, next.js, css, typescript, react, adobe xd, material ui, figma, react.js</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -953,38 +953,46 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18-ResumeMuhammadTahaYasin.pdf</t>
+          <t>23-ResumeSamiUllah3y.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>About Me</t>
+          <t>Sami Ullah Khan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>mtahayasin07@gmail.com</t>
+          <t>samikhaan7814@gmail.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>03406991719</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+          <t>+923443777814</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/sami-khan-111678169</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://github.com/mr-samikhan</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>html, github, css, yarn, tailwind css, react.js, bootstrap, figma, vite, javascript, chrome devtools, git, react, npm</t>
+          <t>github, tailwind css, api's integration, bootstrap, vercel, react, redux, css, material ui</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3 years 6 months</t>
+          <t>3 years 0 months</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -993,16 +1001,16 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>BS Software Engineering</t>
+          <t>BS Computer Science</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>date_range via month-name + year-only + year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>76.54000000000001</v>
+        <v>78.45999999999999</v>
       </c>
       <c r="N9" t="n">
         <v>8</v>
@@ -1011,56 +1019,56 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>19-ResumeMuhammadWaqas3y.pdf</t>
+          <t>18-ResumeMuhammadTahaYasin.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Resumemuhammadwaqas3Y</t>
+          <t>About Me</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Mwbkkj@gmail.com</t>
+          <t>mtahayasin07@gmail.com</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>03126318724</t>
+          <t>03406991719</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>html, github, css, state management, redux, react.js, javascript, react</t>
+          <t>github, javascript, tailwind css, git, npm, bootstrap, chrome devtools, vite, yarn, html, react, css, figma, react.js</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>3 years 0 months</t>
+          <t>5 years 6 months</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>3</v>
+        <v>5.5</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>master</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Master of Management Science (Finance-18 year edu) from IMSciences, Hayatabad</t>
+          <t>BS Software Engineering</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via month-name + year-only + year-only + year-only-fuzzy</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>73.45999999999999</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="N10" t="n">
         <v>9</v>
@@ -1069,64 +1077,56 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>27-Hamza Hamid 3y+.pdf</t>
+          <t>19-ResumeMuhammadWaqas3y.pdf</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hamza Hamid</t>
+          <t>Resumemuhammadwaqas3Y</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>thedev.hamza@gmail.com</t>
+          <t>Mwbkkj@gmail.com</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>03168767587</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/hamxa-hamid/</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>https://github.com/dadhsahb</t>
-        </is>
-      </c>
+          <t>03126318724</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>html, github, jquery, css, tailwind css, react.js, chakra ui, javascript, bootstrap, vue.js, git, react</t>
+          <t>github, javascript, state management, html, react, redux, css, react.js</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2 years 0 months</t>
+          <t>3 years 0 months</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>master</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Bachelor of Science</t>
+          <t>Master of Management Science (Finance-18 year edu) from IMSciences, Hayatabad</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>date_range via mm/yyyy + year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>71.54000000000001</v>
+        <v>73.45999999999999</v>
       </c>
       <c r="N11" t="n">
         <v>10</v>
@@ -1135,29 +1135,29 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>15-ResumeMuhammadLihaz2y.pdf</t>
+          <t>12-ResumeIjlalSHAH-2y.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Muhammad Lihaz Ali</t>
+          <t>Ijlal Shah</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>lehazalil23@gmail.com</t>
+          <t>ijlalshahzr@gmail.com</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>03488899315</t>
+          <t>+923181669799</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>responsive design, html, material ui, css, tailwind css, next.js, react.js, javascript, typescript, react</t>
+          <t>javascript, state management, git, bootstrap, redux toolkit, react hooks, context api, html, angular, react, jquery, redux, typescript, lazy loading, css, material ui, react.js</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>BS Software Engineering Jan 2020 - Feb 2024</t>
+          <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1184,7 +1184,7 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>69.62</v>
+        <v>72.69</v>
       </c>
       <c r="N12" t="n">
         <v>11</v>
@@ -1193,46 +1193,46 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>10-ResumeAQIBZAIB-2y.pdf</t>
+          <t>27-Hamza Hamid 3y+.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Aqib Zaib</t>
+          <t>Hamza Hamid</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>chaqib4u@gmail.com</t>
+          <t>thedev.hamza@gmail.com</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>+923040505345</t>
+          <t>03168767587</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/aqib-zaib-</t>
+          <t>https://www.linkedin.com/in/hamxa-hamid/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://github.com/aqibzaib</t>
+          <t>https://github.com/dadhsahb</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>github, css, tailwind css, vercel, next.js, redux, react.js, react query, redux toolkit, figma, javascript, vue.js, git, react</t>
+          <t>github, javascript, chakra ui, tailwind css, git, bootstrap, css, html, react, jquery, vue.js, react.js</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1 years 6 months</t>
+          <t>1 years 11 months</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>BS SOFTWARE</t>
+          <t>Bachelor of Science</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1250,7 +1250,7 @@
         </is>
       </c>
       <c r="M13" t="n">
-        <v>66.54000000000001</v>
+        <v>70.70999999999999</v>
       </c>
       <c r="N13" t="n">
         <v>12</v>
@@ -1259,47 +1259,47 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Rahul_Mishra_Resume_09-08-2022-16-00-15.pdf</t>
+          <t>15-ResumeMuhammadLihaz2y.pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Rahul Mishra</t>
+          <t>Muhammad Lihaz Ali</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>rahul.mishra@gmail.com</t>
+          <t>lehazalil23@gmail.com</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9876543210</t>
+          <t>03488899315</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>github, rest api, bitbucket, javascript, bootstrap, git</t>
+          <t>javascript, tailwind css, next.js, responsive design, html, typescript, react, css, material ui, react.js</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>4 years 0 months</t>
+          <t>2 years 0 months</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>master</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Master of Computer Applications, National Institute of Technology Allahabad (MNNIT), U.P</t>
+          <t>BS Software Engineering Jan 2020 - Feb 2024</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1308,7 +1308,7 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>64.23</v>
+        <v>69.62</v>
       </c>
       <c r="N14" t="n">
         <v>13</v>
@@ -1317,56 +1317,64 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Shubham_Mishra_Resume_09-08-2022-16-16-14.pdf</t>
+          <t>10-ResumeAQIBZAIB-2y.pdf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Shubham Mishra</t>
+          <t>Aqib Zaib</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>shubham.mishra@gmail.com</t>
+          <t>chaqib4u@gmail.com</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9876543210</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+          <t>+923040505345</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/aqib-zaib-</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://github.com/aqibzaib</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>github, rest api, bitbucket, javascript, bootstrap, git</t>
+          <t>github, javascript, tailwind css, git, css, redux toolkit, next.js, react query, react, vercel, redux, vue.js, figma, react.js</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>3 years 0 months</t>
+          <t>1 years 6 months</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>master</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Master of Computer Applications</t>
+          <t>BS SOFTWARE</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via mm/yyyy + year-only</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>64.23</v>
+        <v>66.54000000000001</v>
       </c>
       <c r="N15" t="n">
         <v>14</v>
@@ -1375,51 +1383,47 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>11-ResumeEJAZAHMAD.pdf</t>
+          <t>Shubham_Mishra_Resume_09-08-2022-16-16-14.pdf</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ejaz Ahmad</t>
+          <t>Shubham Mishra</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ayanejaz420fwisg_dpy@indeedemail.com</t>
+          <t>shubham.mishra@gmail.com</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>+923313322420</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/in/ejaz-ahmad-2359a2247</t>
-        </is>
-      </c>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>less, html, css, rest api, graphql, typescript, react</t>
+          <t>github, javascript, git, bootstrap, bitbucket, rest api</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2 years 0 months</t>
+          <t>3 years 0 months</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>master</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Bachelor / No major degree found but there is a university mention</t>
+          <t>Master of Computer Applications</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1428,7 +1432,7 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>63.38</v>
+        <v>64.23</v>
       </c>
       <c r="N16" t="n">
         <v>15</v>
@@ -1437,64 +1441,56 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>7-Muhammad Yasin - Software Engineer.pdf</t>
+          <t>Rahul_Mishra_Resume_09-08-2022-16-00-15.pdf</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Muhammad Yasin Software Engineer</t>
+          <t>Rahul Mishra</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>yasinwaheed11@gmail.com</t>
+          <t>rahul.mishra@gmail.com</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>+923026770777</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/yasinwahid111</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>https://github.com/YasinWahid</t>
-        </is>
-      </c>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>responsive design, html, github, angular, css, react.js, figma, javascript, bootstrap, git, typescript, react</t>
+          <t>github, javascript, git, bootstrap, bitbucket, rest api</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1 years 2 months</t>
+          <t>4 years 0 months</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>1.2</v>
+        <v>4</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>master</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Hifah Technologies | Abbottabad Bachelor of Software Engineering</t>
+          <t>Master of Computer Applications, National Institute of Technology Allahabad (MNNIT), U.P</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M17" t="n">
-        <v>63.21</v>
+        <v>64.23</v>
       </c>
       <c r="N17" t="n">
         <v>16</v>
@@ -1503,56 +1499,60 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>24-ResumeTayyabHussainshah.pdf</t>
+          <t>17-ResumeMuhammadShayan3y.pdf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tayyab Hussain Shah</t>
+          <t>Muhammad Shayan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>tayabsajid5@gmail.com</t>
+          <t>kshayan091@gmail.com</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>+923365298230</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
+          <t>+923168104861</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/shayan-khan20</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>github, angular, css, tailwind css, vercel, sass, next.js, redux, react.js, figma, vite, javascript, git, typescript, react</t>
+          <t>github, javascript, next.js, typescript, react, redux, material ui, figma, seo optimization</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1 years 4 months</t>
+          <t>3 years 0 months</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>1.3</v>
+        <v>3</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>high school</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Software Engineering</t>
+          <t>Higher school January 2020– March 2022</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M18" t="n">
-        <v>62.95</v>
+        <v>63.38</v>
       </c>
       <c r="N18" t="n">
         <v>17</v>
@@ -1561,29 +1561,33 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12-ResumeIjlalSHAH-2y.pdf</t>
+          <t>11-ResumeEJAZAHMAD.pdf</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Ijlal Shah</t>
+          <t>Ejaz Ahmad</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ijlalshahzr@gmail.com</t>
+          <t>ayanejaz420fwisg_dpy@indeedemail.com</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>+923181669799</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
+          <t>+923313322420</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/ejaz-ahmad-2359a2247</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>html, jquery, material ui, css, angular, state management, redux, react.js, redux toolkit, context api, lazy loading, javascript, bootstrap, git, typescript, react, react hooks</t>
+          <t>html, typescript, react, css, rest api, less, graphql</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1596,17 +1600,21 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr"/>
+          <t>bachelor</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Bachelor (inferred) / No major degree found but mentions university</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
       <c r="M19" t="n">
-        <v>62.69</v>
+        <v>63.38</v>
       </c>
       <c r="N19" t="n">
         <v>18</v>
@@ -1615,46 +1623,46 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>22-ResumeSaadAhmad-1y.pdf</t>
+          <t>7-Muhammad Yasin - Software Engineer.pdf</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Saad Ahmad</t>
+          <t>Muhammad Yasin Software Engineer</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>saadahmad6830879@gmail.com</t>
+          <t>yasinwaheed11@gmail.com</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>923176830879</t>
+          <t>+923026770777</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://linkedin.com/in/saadahmad879</t>
+          <t>https://www.linkedin.com/in/yasinwahid111</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://github.com/SaADii09</t>
+          <t>https://github.com/YasinWahid</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>html, github, css, state management, tailwind css, redux, react.js, javascript, git, react</t>
+          <t>github, javascript, git, bootstrap, responsive design, html, angular, react, typescript, css, figma, react.js</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0 years 8 months</t>
+          <t>1 years 2 months</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1663,16 +1671,16 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>BS Computer Science</t>
+          <t>Hifah Technologies | Abbottabad Bachelor of Software Engineering</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
+          <t>date_range via fuzzy-month + month-name + year-only</t>
         </is>
       </c>
       <c r="M20" t="n">
-        <v>61.28</v>
+        <v>63.21</v>
       </c>
       <c r="N20" t="n">
         <v>19</v>
@@ -1681,38 +1689,46 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Shubham_Mishra_Resume_10-08-2022-16-06-13.pdf</t>
+          <t>Data_engineer(Sample 4+ year).pdf</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Shubham Mishra</t>
+          <t>Biswajit Khetan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>shubham.mishra@gmail.com</t>
+          <t>bisjwa1445@gmail.com</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>9876543210</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
+          <t>+91987654321</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/11i/</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://github.com/AnkitDB9</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>github, rest api, bitbucket, git, jenkins</t>
+          <t>github, rest api</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>7 years 0 months</t>
+          <t>4 years 8 months</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>7</v>
+        <v>4.7</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1721,16 +1737,16 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Bachelor of Engineering in Computer Science,</t>
+          <t>Bachelor of Technology,</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only-fuzzy</t>
         </is>
       </c>
       <c r="M21" t="n">
-        <v>61.15</v>
+        <v>63.08</v>
       </c>
       <c r="N21" t="n">
         <v>20</v>
@@ -1739,64 +1755,64 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1-Fahadalamresume.pdf</t>
+          <t>resume_juanjosecarin.pdf</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Fahad Alam</t>
+          <t>Juan Jose Carin</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>fahadalam12405@gmail.com</t>
+          <t>juanjose.carin@gmail.com</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>+923272748498</t>
+          <t>940416503364590</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/fahad-alam</t>
+          <t>https://linkedin.com/in/juanjosecarin</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://github.com/Fahad12405</t>
+          <t>https://github.com/juanjocarin/W261-Machine-Learning-At-Scale/blob/master/Week07-MrJob/MIDS-W261-2015-HWK-Week07-CarinLlopSatpati-groupZ.ipynb</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>redux, javascript, react, html, next.js, postcss, github, jquery, state management, tailwind css, axios, vue.js, git, typescript, webpack, css, react.js, redux toolkit, context api, vite, bootstrap</t>
+          <t>github, git</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1 years 3 months</t>
+          <t>5 years 1 months</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>1.2</v>
+        <v>5.1</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>high school</t>
+          <t>master</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Intermediate, Cs</t>
+          <t>Master of Information and Data Science</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>date_range via reverse-order</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only-fuzzy</t>
         </is>
       </c>
       <c r="M22" t="n">
-        <v>60.19</v>
+        <v>63.08</v>
       </c>
       <c r="N22" t="n">
         <v>21</v>
@@ -1805,42 +1821,38 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Nezuko_Kamado_Resume_10-08-2022-16-04-20.pdf</t>
+          <t>24-ResumeTayyabHussainshah.pdf</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kamado Associate Lead</t>
+          <t>Tayyab Hussain Shah</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>hello.ineuron@gmail.com</t>
+          <t>tayabsajid5@gmail.com</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>9923312341</t>
+          <t>+923365298230</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>https://github.com/model</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>rest api, github</t>
+          <t>github, javascript, tailwind css, git, vite, next.js, angular, react, sass, redux, vercel, typescript, css, figma, react.js</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>6 years 0 months</t>
+          <t>1 years 4 months</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>6</v>
+        <v>1.3</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1849,16 +1861,16 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Bachelor Of Technology in Computer Science</t>
+          <t>Bachelor of Science in Software Engineering</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
       <c r="M23" t="n">
-        <v>60.08</v>
+        <v>62.95</v>
       </c>
       <c r="N23" t="n">
         <v>22</v>
@@ -1867,55 +1879,55 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2-TouseefAbidCv.pdf</t>
+          <t>22-ResumeSaadAhmad-1y.pdf</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Touseef Abid</t>
+          <t>Saad Ahmad</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>touseefabid737@gmail.com</t>
+          <t>saadahmad6830879@gmail.com</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>+923102939875</t>
+          <t>923176830879</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/touseefabid</t>
+          <t>https://linkedin.com/in/saadahmad879</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://github.com/Touseef4705</t>
+          <t>https://github.com/SaADii09</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>html, github, css, yarn, vercel, next.js, redux, react.js, redux toolkit, javascript, git, react router, react, npm</t>
+          <t>github, javascript, state management, tailwind css, git, html, react, redux, css, react.js</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1 years 6 months</t>
+          <t>0 years 8 months</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>1.5</v>
+        <v>0.7</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>high school</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Intermediate, Business Commerce</t>
+          <t>BS Computer Science</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -1924,7 +1936,7 @@
         </is>
       </c>
       <c r="M24" t="n">
-        <v>59.62</v>
+        <v>61.28</v>
       </c>
       <c r="N24" t="n">
         <v>23</v>
@@ -1933,46 +1945,38 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MAqeel.pdf</t>
+          <t>Shubham_Mishra_Resume_10-08-2022-16-06-13.pdf</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Muhammad Aqeel</t>
+          <t>Shubham Mishra</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>maqeelcs09@gmail.com</t>
+          <t>shubham.mishra@gmail.com</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>+923419905547</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/in/aqeelkhan09</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>https://github.com/maqeel019</t>
-        </is>
-      </c>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>html, github, css, javascript, git</t>
+          <t>github, git, jenkins, bitbucket, rest api</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1 years 6 months</t>
+          <t>7 years 0 months</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>1.5</v>
+        <v>7</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -1981,16 +1985,16 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Bachelor of Computer Science</t>
+          <t>Bachelor of Engineering in Computer Science,</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M25" t="n">
-        <v>57.31</v>
+        <v>61.15</v>
       </c>
       <c r="N25" t="n">
         <v>24</v>
@@ -1999,64 +2003,64 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ScholarCV.pdf</t>
+          <t>1-Fahadalamresume.pdf</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Muhammad Aqeel</t>
+          <t>Fahad Alam</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>maqeelcs09@gmail.com</t>
+          <t>fahadalam12405@gmail.com</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>+923419905547</t>
+          <t>+923272748498</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://linkedin.com/in/aqeelkhan09</t>
+          <t>https://www.linkedin.com/in/fahad-alam</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://github.com/maqeel019</t>
+          <t>https://github.com/Fahad12405</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>html, github, css, javascript, git</t>
+          <t>state management, bootstrap, redux toolkit, context api, react, webpack, javascript, postcss, git, next.js, html, jquery, css, vite, redux, vue.js, github, tailwind css, axios, typescript, react.js</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1 years 6 months</t>
+          <t>1 years 3 months</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>high school</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Bachelor of Computer Science</t>
+          <t>Intermediate, Cs</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
+          <t>date_range via reverse-order</t>
         </is>
       </c>
       <c r="M26" t="n">
-        <v>57.31</v>
+        <v>60.19</v>
       </c>
       <c r="N26" t="n">
         <v>25</v>
@@ -2065,46 +2069,42 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Data_engineer(Sample 4+ year).pdf</t>
+          <t>Nezuko_Kamado_Resume_10-08-2022-16-04-20.pdf</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Biswajit Khetan</t>
+          <t>Kamado Associate Lead</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>bisjwa1445@gmail.com</t>
+          <t>hello.ineuron@gmail.com</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>+91987654321</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/11i/</t>
-        </is>
-      </c>
+          <t>9923312341</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://github.com/AnkitDB9</t>
+          <t>https://github.com/model</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>rest api, github</t>
+          <t>github, rest api</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2 years 5 months</t>
+          <t>6 years 0 months</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>2.4</v>
+        <v>6</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -2113,16 +2113,16 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Bachelor of Technology,</t>
+          <t>Bachelor Of Technology in Computer Science</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M27" t="n">
-        <v>57.24</v>
+        <v>60.08</v>
       </c>
       <c r="N27" t="n">
         <v>26</v>
@@ -2131,60 +2131,64 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Naruto_uzumaki_Resume_10-08-2022-15-31-44.pdf</t>
+          <t>2-TouseefAbidCv.pdf</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Naruto Uzumaki</t>
+          <t>Touseef Abid</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>hello.ineuron@gmail.com</t>
+          <t>touseefabid737@gmail.com</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>9923312341</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
+          <t>+923102939875</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/touseefabid</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://github.com/PROFILE</t>
+          <t>https://github.com/Touseef4705</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>github</t>
+          <t>github, javascript, git, npm, redux toolkit, next.js, yarn, html, react, vercel, redux, css, react.js, react router</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>4 years 0 months</t>
+          <t>1 years 6 months</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>high school</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Bachelor Of Technology in Computer Science, Jaypee Institute Of Information Technology</t>
+          <t>Intermediate, Business Commerce</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
       <c r="M28" t="n">
-        <v>57</v>
+        <v>59.62</v>
       </c>
       <c r="N28" t="n">
         <v>27</v>
@@ -2193,34 +2197,46 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Tanjiro_Bhatia_Resume_09-08-2022-19-15-13.pdf</t>
+          <t>16-ResumeMuhammadluqmanKhan1y+.pdf</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Tanjiro Bhatia</t>
+          <t>Muhammad Luqman</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tanjiro.bhatia67@gmail.com</t>
+          <t>IK3281751@gmail.com</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>9923312341</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
+          <t>+923361935561</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/muhammad-luqman-khan-051047267</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://github.com/Luqmanoffical</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>github, javascript, bootstrap, html, typescript, react, css, figma, react.js, netlify</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>6 years 0 months</t>
+          <t>1 years 0 months</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -2229,16 +2245,16 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Bachelor / No major degree found but there is a university mention</t>
+          <t>Bachelor's Degree in Information Technology</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via year-only + year-only-fuzzy</t>
         </is>
       </c>
       <c r="M29" t="n">
-        <v>55</v>
+        <v>58.46</v>
       </c>
       <c r="N29" t="n">
         <v>28</v>
@@ -2247,42 +2263,46 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>21-ResumeRehmanZeb2y+.pdf</t>
+          <t>ScholarCV.pdf</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Resumerehmanzeb2Y+</t>
+          <t>Muhammad Aqeel</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>rehmanzeb2k17@gmail.com</t>
+          <t>maqeelcs09@gmail.com</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>+923119449029</t>
+          <t>+923419905547</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/rehmanzeb</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
+          <t>https://linkedin.com/in/aqeelkhan09</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://github.com/maqeel019</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>responsive design, css, tailwind css, next.js, react.js, javascript, bootstrap, git, react</t>
+          <t>github, javascript, git, html, css</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>0 years 9 months</t>
+          <t>1 years 6 months</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -2291,16 +2311,16 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>BS Computer Science</t>
+          <t>Bachelor of Computer Science</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + month-only + year</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
       <c r="M30" t="n">
-        <v>53.96</v>
+        <v>57.31</v>
       </c>
       <c r="N30" t="n">
         <v>29</v>
@@ -2309,56 +2329,64 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>17-ResumeMuhammadShayan3y.pdf</t>
+          <t>MAqeel.pdf</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Muhammad Shayan</t>
+          <t>Muhammad Aqeel</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>kshayan091@gmail.com</t>
+          <t>maqeelcs09@gmail.com</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>+923168104861</t>
+          <t>+923419905547</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/shayan-khan20</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
+          <t>https://linkedin.com/in/aqeelkhan09</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://github.com/maqeel019</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>github, material ui, next.js, redux, seo optimization, figma, javascript, typescript, react</t>
+          <t>github, javascript, git, html, css</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1 years 11 months</t>
+          <t>1 years 6 months</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr"/>
+          <t>bachelor</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Bachelor of Computer Science</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
       <c r="M31" t="n">
-        <v>52.55</v>
+        <v>57.31</v>
       </c>
       <c r="N31" t="n">
         <v>30</v>
@@ -2367,30 +2395,42 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>data-scientist-resume-sample-template.pdf</t>
+          <t>Naruto_uzumaki_Resume_10-08-2022-15-31-44.pdf</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Robin Doe</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
+          <t>Naruto Uzumaki</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>hello.ineuron@gmail.com</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>123451234567090</t>
+          <t>9923312341</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://github.com/PROFILE</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>github</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>8 years 6 months</t>
+          <t>4 years 0 months</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>8.5</v>
+        <v>4</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -2399,16 +2439,16 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>ba Eng al) - AMT</t>
+          <t>Bachelor Of Technology in Computer Science, Jaypee Institute Of Information Technology</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>date_range via year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M32" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="N32" t="n">
         <v>31</v>
@@ -2417,38 +2457,42 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>20-ResumeRAJAABDULLAH1.5y.pdf</t>
+          <t>3-AJSwatiResume.pdf</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Raja Abdullah</t>
+          <t>Abdullah Javed</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>rabdullah806@gmail.com</t>
+          <t>abdullah.javed9438@gmail.com</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>923175510676</t>
+          <t>+923499377144</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://github.com/AbdullahKhanSwati</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>html, css, javascript</t>
+          <t>github, javascript, state management, tailwind css, react hooks, responsive design, react, jquery, redux, lazy loading, css, react.js, netlify</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1 years 6 months</t>
+          <t>1 years 0 months</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -2457,16 +2501,16 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Bachelor / No major degree found but there is a university mention</t>
+          <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via year-only-fuzzy</t>
         </is>
       </c>
       <c r="M33" t="n">
-        <v>49.23</v>
+        <v>55.46</v>
       </c>
       <c r="N33" t="n">
         <v>32</v>
@@ -2475,46 +2519,34 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>23-ResumeSamiUllah3y.pdf</t>
+          <t>Tanjiro_Bhatia_Resume_09-08-2022-19-15-13.pdf</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Sami Ullah Khan</t>
+          <t>Tanjiro Bhatia</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>samikhaan7814@gmail.com</t>
+          <t>Tanjiro.bhatia67@gmail.com</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>+923443777814</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/in/sami-khan-111678169</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>https://github.com/mr-samikhan</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>api's integration, github, material ui, css, tailwind css, vercel, redux, bootstrap, react</t>
-        </is>
-      </c>
+          <t>9923312341</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
-          <t>0 years 0 months</t>
+          <t>6 years 0 months</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -2523,16 +2555,16 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>BS Computer Science</t>
+          <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>none via none</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M34" t="n">
-        <v>48.46</v>
+        <v>55</v>
       </c>
       <c r="N34" t="n">
         <v>33</v>
@@ -2541,46 +2573,42 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16-ResumeMuhammadluqmanKhan1y+.pdf</t>
+          <t>21-ResumeRehmanZeb2y+.pdf</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Muhammad Luqman</t>
+          <t>Resumerehmanzeb2Y+</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>IK3281751@gmail.com</t>
+          <t>rehmanzeb2k17@gmail.com</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>+923361935561</t>
+          <t>+923119449029</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://linkedin.com/in/muhammad-luqman-khan-051047267</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>https://github.com/Luqmanoffical</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/in/rehmanzeb</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>html, github, css, netlify, react.js, figma, javascript, bootstrap, typescript, react</t>
+          <t>javascript, tailwind css, git, bootstrap, next.js, responsive design, react, css, react.js</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>0 years 0 months</t>
+          <t>0 years 9 months</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
@@ -2589,16 +2617,16 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Bachelor's Degree in Information Technology</t>
+          <t>BS Computer Science</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>none via none</t>
+          <t>date_range via fuzzy-month + month-name + year-only + month-only + year</t>
         </is>
       </c>
       <c r="M35" t="n">
-        <v>48.46</v>
+        <v>53.96</v>
       </c>
       <c r="N35" t="n">
         <v>34</v>
@@ -2607,64 +2635,48 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5-JAWADRESUME.pdf</t>
+          <t>data-scientist-resume-sample-template.pdf</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Jawad Ali</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>jawadalikhan359@gmail.com</t>
-        </is>
-      </c>
+          <t>Robin Doe</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>03139908709</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/jawadali1535</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>https://github.com/JawadAli1535</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>github, jquery, css, tailwind css, vercel, sass, axios, redux, javascript, git, typescript, react</t>
-        </is>
-      </c>
+          <t>123451234567090</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>0 years 5 months</t>
+          <t>8 years 6 months</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>0.4</v>
+        <v>8.5</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>high school</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Nodejs(intermediate)</t>
+          <t>ba Eng al) - AMT</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only</t>
+          <t>date_range via year-only + year-only-fuzzy</t>
         </is>
       </c>
       <c r="M36" t="n">
-        <v>45.71</v>
+        <v>52</v>
       </c>
       <c r="N36" t="n">
         <v>35</v>
@@ -2673,34 +2685,38 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Riya_Bhatiya_Resume_09-08-2022-19-26-53.pdf</t>
+          <t>20-ResumeRAJAABDULLAH1.5y.pdf</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Riya Bhatiya</t>
+          <t>Raja Abdullah</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>riya.bhatia67@gmail.com</t>
+          <t>rabdullah806@gmail.com</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>9923312341</t>
+          <t>923175510676</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>html, javascript, css</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2 years 0 months</t>
+          <t>1 years 6 months</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -2709,7 +2725,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Bachelor Of Technology in Computer Science Freelance Mentor Of Data Structure and Algorithms</t>
+          <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -2718,7 +2734,7 @@
         </is>
       </c>
       <c r="M37" t="n">
-        <v>45</v>
+        <v>49.23</v>
       </c>
       <c r="N37" t="n">
         <v>36</v>
@@ -2727,64 +2743,60 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>resume_juanjosecarin.pdf</t>
+          <t>Nitish Kumar.pdf</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Juan Jose Carin</t>
+          <t>Nitish Kumar</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>juanjose.carin@gmail.com</t>
+          <t>xyz@gmail.com</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>940416503364590</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/in/juanjosecarin</t>
-        </is>
-      </c>
+          <t>9977141714</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://github.com/juanjocarin/W261-Machine-Learning-At-Scale/blob/master/Week07-MrJob/MIDS-W261-2015-HWK-Week07-CarinLlopSatpati-groupZ.ipynb</t>
+          <t>https://github.com/vishalsingh17</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>github, git</t>
+          <t>html, css, git, github</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1 years 2 months</t>
+          <t>1 years 0 months</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>master</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Master of Information and Data Science</t>
+          <t>12/2015 – 12/2018 BCA</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M38" t="n">
-        <v>44.74</v>
+        <v>46.23</v>
       </c>
       <c r="N38" t="n">
         <v>37</v>
@@ -2793,60 +2805,64 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Shankar_chavan_Resume_10-08-2022-12-54-00.pdf</t>
+          <t>5-JAWADRESUME.pdf</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Shankar Chavan</t>
+          <t>Jawad Ali</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>shankar.chavan@gmail.com</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
+          <t>jawadalikhan359@gmail.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>03139908709</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/</t>
+          <t>https://www.linkedin.com/in/jawadali1535</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://github.com/</t>
+          <t>https://github.com/JawadAli1535</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>github</t>
+          <t>github, javascript, tailwind css, git, axios, sass, react, vercel, redux, jquery, typescript, css</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1 years 6 months</t>
+          <t>0 years 5 months</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.5</v>
+        <v>0.4</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>master</t>
+          <t>high school</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Master Degree, SPPU University</t>
+          <t>Nodejs(intermediate)</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via fuzzy-month + month-name + year-only</t>
         </is>
       </c>
       <c r="M39" t="n">
-        <v>43</v>
+        <v>45.71</v>
       </c>
       <c r="N39" t="n">
         <v>38</v>
@@ -2855,42 +2871,34 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>26-Sameer Khan Cv3y.pdf</t>
+          <t>Riya_Bhatiya_Resume_09-08-2022-19-26-53.pdf</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Sameer Khan</t>
+          <t>Riya Bhatiya</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>berlanjan123@gmail.com</t>
+          <t>riya.bhatia67@gmail.com</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>+923169769253</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/sameer-khan-660966251</t>
-        </is>
-      </c>
+          <t>9923312341</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>html, github, css, next.js, bootstrap, react</t>
-        </is>
-      </c>
+      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>0 years 0 months</t>
+          <t>2 years 0 months</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -2899,16 +2907,16 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Degree Bs Computer Science</t>
+          <t>Bachelor Of Technology in Computer Science Freelance Mentor Of Data Structure and Algorithms</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>none via none</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M40" t="n">
-        <v>37.23</v>
+        <v>45</v>
       </c>
       <c r="N40" t="n">
         <v>39</v>
@@ -2917,56 +2925,60 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Nitish Kumar.pdf</t>
+          <t>Shankar_chavan_Resume_10-08-2022-12-54-00.pdf</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Nitish Kumar</t>
+          <t>Shankar Chavan</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>xyz@gmail.com</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>9977141714</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr"/>
+          <t>shankar.chavan@gmail.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://github.com/vishalsingh17</t>
+          <t>https://github.com/</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>html, github, git, css</t>
+          <t>github</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1 years 0 months</t>
+          <t>1 years 6 months</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr"/>
+          <t>master</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Master Degree, SPPU University</t>
+        </is>
+      </c>
       <c r="L41" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
       <c r="M41" t="n">
-        <v>36.23</v>
+        <v>43</v>
       </c>
       <c r="N41" t="n">
         <v>40</v>
@@ -2975,33 +2987,33 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>3-AJSwatiResume.pdf</t>
+          <t>26-Sameer Khan Cv3y.pdf</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Abdullah Javed</t>
+          <t>Sameer Khan</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>abdullah.javed9438@gmail.com</t>
+          <t>berlanjan123@gmail.com</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>+923499377144</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>https://github.com/AbdullahKhanSwati</t>
-        </is>
-      </c>
+          <t>+923169769253</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sameer-khan-660966251</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>responsive design, github, jquery, css, state management, tailwind css, netlify, redux, react.js, lazy loading, javascript, react, react hooks</t>
+          <t>github, bootstrap, next.js, html, react, css</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3014,17 +3026,21 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr"/>
+          <t>bachelor</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Degree Bs Computer Science</t>
+        </is>
+      </c>
       <c r="L42" t="inlineStr">
         <is>
           <t>none via none</t>
         </is>
       </c>
       <c r="M42" t="n">
-        <v>35.46</v>
+        <v>37.23</v>
       </c>
       <c r="N42" t="n">
         <v>41</v>
@@ -3127,7 +3143,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>BACHELOR OF SCIENCE University of Swabi</t>
+          <t>muhammad abu aqeel nationality: pakistani gender: male phone number: (+92) 3419905547 (mobile) email address: maqeelcs09@gmail.com address: pakistan (home) about me a dedicated individual with a proven track record of achieving and exceeding goals through unwavering determination and a commitment to excellence education and training lahore, pakistan bachelor of science university of swabi field of studycomputer science 2020 bam khel,swabi, pakistan intermediate the glorious college of science &amp; technology language skills mother tongue(s): urdu | pashto other language(s): understanding speaking writing spoken spoken listening reading production interaction english c1 c1 c1 c1 c1 levels: a1 and a2: basic user; b1 and b2: independent user; c1 and c2: proficient user additional information management and leadership skills skills strategic planning and execution: • proficient in developing long-term strategies and effectively executing action plans to achieve organizational goals. • skilled at aligning business objectives with actionable plans for efficient resource utilization. team leadership and motivation: • proven ability to lead and inspire teams, fostering a collaborative and high-performing work environment. • experienced in setting clear expectations, providing constructive feedback, and empowering team members to reach their potential. decision making and problem-solving: • strong analytical and critical thinking skills, enabling effective decision-making in complex situations.</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">

</xml_diff>

<commit_message>
Refactor: Moved config & skill sets to /config, updated imports & paths
</commit_message>
<xml_diff>
--- a/output/all_candidates_ranked.xlsx
+++ b/output/all_candidates_ranked.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -503,46 +503,46 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>25-Resumezeeshanzahoor3y+.pdf</t>
+          <t>13-ResumeMominKhan 4y.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Zeeshan Zahoor</t>
+          <t>Momin Hyat Khan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>zeeshanzahoor409@gmail.com</t>
+          <t>mominhyatkhandeveloper@gmail.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+923421905266</t>
+          <t>03345674415</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/zeeshan-zahoor-220b0b130</t>
+          <t>https://linkedin.com/in/mominhyatkhan</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://github.com/zeeshanshaanu</t>
+          <t>https://github.com/mominhyatkhan</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>bootstrap, redux toolkit, react, material ui, javascript, git, next.js, css, websockets, netlify, redux, figma, github, tailwind css, responsive design, typescript, vercel, lighthouse, react.js</t>
+          <t>eslint, oauth, integration testing, jwt, mysql, hive, agile, react, typescript, nest.js, tailwind css, github, monitoring, spring, spring boot, java, authorization, css, redux, unit testing, authentication, javascript, html, axios, next.js, material ui, git, react query, prettier</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3 years 0 months</t>
+          <t>4 years 0 months</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -551,7 +551,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>🎓 BS in Computer Science (2016 – 2020) | Gov’t Post Graduate College, Haripur</t>
+          <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -569,46 +569,46 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13-ResumeMominKhan 4y.pdf</t>
+          <t>28-zeeshaan updated4y+.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Momin Hyat Khan</t>
+          <t>Zeeshan Zahoor</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>mominhyatkhandeveloper@gmail.com</t>
+          <t>zeeshanzahoor409@gmail.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>03345674415</t>
+          <t>+923421905266</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://linkedin.com/in/mominhyatkhan</t>
+          <t>https://www.linkedin.com/in/zeeshan-zahoor-220b0b130</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://github.com/mominhyatkhan</t>
+          <t>https://github.com/zeeshanshaanu</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>github, javascript, prettier, eslint, tailwind css, git, next.js, html, axios, react query, react, typescript, redux, css, material ui</t>
+          <t>responsive design, react.js, figma, react, node.js, typescript, netlify, tailwind css, github, vs code, vercel, css, redux, authentication, communication, websockets, javascript, redux toolkit, next.js, lighthouse, material ui, git, data visualization, bootstrap, mongodb, express</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>4 years 0 months</t>
+          <t>3 years 0 months</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -617,7 +617,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Bachelor (inferred) / No major degree found but mentions university</t>
+          <t>🎓 BS in Computer Science (2016 – 2020) | Gov’t Post Graduate College, Haripur</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>28-zeeshaan updated4y+.pdf</t>
+          <t>25-Resumezeeshanzahoor3y+.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>bootstrap, redux toolkit, react, material ui, javascript, git, next.js, css, websockets, netlify, redux, figma, github, tailwind css, responsive design, typescript, vercel, lighthouse, react.js</t>
+          <t>responsive design, react.js, figma, react, node.js, typescript, netlify, tailwind css, github, vs code, vercel, css, redux, authentication, communication, websockets, javascript, redux toolkit, next.js, lighthouse, material ui, git, data visualization, bootstrap, mongodb, express</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>progressive web apps, jest, state management, react, webpack, javascript, git, next.js, code splitting, css, netlify, graphql, github actions, single page applications, redux, react testing library, vue.js, figma, babel, github, tailwind css, responsive design, cypress, typescript, vercel, lazy loading, styled components, seo optimization, react.js</t>
+          <t>postgresql, vue.js, graphql, responsive design, react.js, figma, cypress, docker, agile, single page applications, react, styled components, node.js, typescript, lazy loading, netlify, tailwind css, github, vercel, github actions, webpack, scrum, css, redux, progressive web apps, aws, seo optimization, javascript, next.js, babel, code splitting, state management, react testing library, git, jest, mongodb, express</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -767,46 +767,42 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4-AyazKhan-Software Engineer-4y.pdf</t>
+          <t>ResumeAbdullahKhan.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ayaz Khan</t>
+          <t>Resumeabdullahkhan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pakistan03479@gmail.com</t>
+          <t>abdullahkh1144@gmail.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>+923139131611</t>
+          <t>+923105778487</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://linkedin.com/in/ayazcoder</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>https://github.com/ayazcoder</t>
-        </is>
-      </c>
+          <t>https://linkedin.com/in/abdullah-khan-0727b0247</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>github, javascript, tailwind css, git, react hooks, github actions, react, css, material ui, react.js</t>
+          <t>graphql, responsive design, react.js, agile, firebase, react, node.js, typescript, azure, tailwind css, css, redux, unit testing, authentication, communication, websockets, aws, javascript, seo optimization, project management, next.js, git, bootstrap, mongodb</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>3 years 2 months</t>
+          <t>5 years 0 months</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -815,16 +811,16 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Bachelor of Software Engineering</t>
+          <t>Bachelor of Science in SOFTWARE ENGINEERING</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>81.54000000000001</v>
+        <v>82.62</v>
       </c>
       <c r="N6" t="n">
         <v>5</v>
@@ -833,42 +829,46 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>9-Raja Saqib Resume 2.5y.pdf</t>
+          <t>4-AyazKhan-Software Engineer-4y.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Saqib Iftikhar</t>
+          <t>Ayaz Khan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>saqibifitkhar756@gmail.com</t>
+          <t>pakistan03479@gmail.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>03403118722</t>
+          <t>+923139131611</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/saqib--iftikhar</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>https://linkedin.com/in/ayazcoder</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://github.com/ayazcoder</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>javascript, state management, tailwind css, git, html, react, redux, css, material ui, figma, react.js</t>
+          <t>react.js, python, mysql, react hooks, firebase, react, node.js, ios, azure, tailwind css, github, github actions, scrum, css, communication, android, javascript, project management, flutter, material ui, git, mongodb, express</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2 years 6 months</t>
+          <t>3 years 2 months</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -877,16 +877,16 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>BS (COMPUTER SCIENCE) ( 2018 - 2022 )</t>
+          <t>Bachelor of Software Engineering</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>80.69</v>
+        <v>81.54000000000001</v>
       </c>
       <c r="N7" t="n">
         <v>6</v>
@@ -895,38 +895,42 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6-JUNAID AKBAR 3y.pdf</t>
+          <t>9-Raja Saqib Resume 2.5y.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Junaid Akbar</t>
+          <t>Saqib Iftikhar</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>junaidjojo4@gmail.com</t>
+          <t>saqibifitkhar756@gmail.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>+923337661597</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+          <t>03403118722</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/saqib--iftikhar</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>github, javascript, tailwind css, git, bootstrap, next.js, css, typescript, react, adobe xd, material ui, figma, react.js</t>
+          <t>react.js, figma, mysql, agile, react, node.js, r, tailwind css, authorization, css, redux, laravel, authentication, communication, javascript, html, state management, material ui, git, mongodb, express</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>3 years 0 months</t>
+          <t>2 years 6 months</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -935,7 +939,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Software Engineering</t>
+          <t>BS (COMPUTER SCIENCE) ( 2018 - 2022 )</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -944,7 +948,7 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>79.62</v>
+        <v>80.69</v>
       </c>
       <c r="N8" t="n">
         <v>7</v>
@@ -953,37 +957,29 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>23-ResumeSamiUllah3y.pdf</t>
+          <t>6-JUNAID AKBAR 3y.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Sami Ullah Khan</t>
+          <t>Junaid Akbar</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>samikhaan7814@gmail.com</t>
+          <t>junaidjojo4@gmail.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>+923443777814</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/in/sami-khan-111678169</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>https://github.com/mr-samikhan</t>
-        </is>
-      </c>
+          <t>+923337661597</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>github, tailwind css, api's integration, bootstrap, vercel, react, redux, css, material ui</t>
+          <t>next.js, react, react.js, figma, typescript, material ui, css, git, bootstrap, adobe xd, tailwind css, github, javascript, linux</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1001,7 +997,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>BS Computer Science</t>
+          <t>Bachelor of Science in Software Engineering</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1010,7 +1006,7 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>78.45999999999999</v>
+        <v>79.62</v>
       </c>
       <c r="N9" t="n">
         <v>8</v>
@@ -1019,38 +1015,46 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18-ResumeMuhammadTahaYasin.pdf</t>
+          <t>23-ResumeSamiUllah3y.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>About Me</t>
+          <t>Sami Ullah Khan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>mtahayasin07@gmail.com</t>
+          <t>samikhaan7814@gmail.com</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>03406991719</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+          <t>+923443777814</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/sami-khan-111678169</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://github.com/mr-samikhan</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>github, javascript, tailwind css, git, npm, bootstrap, chrome devtools, vite, yarn, html, react, css, figma, react.js</t>
+          <t>api's integration, firebase, react, azure, machine learning, css, vercel, redux, material ui, docker, tailwind css, github, php, bootstrap, aws, mongodb, express</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>5 years 6 months</t>
+          <t>3 years 0 months</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>5.5</v>
+        <v>3</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1059,16 +1063,16 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>BS Software Engineering</t>
+          <t>BS Computer Science</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>date_range via month-name + year-only + year-only + year-only-fuzzy</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>76.54000000000001</v>
+        <v>78.45999999999999</v>
       </c>
       <c r="N10" t="n">
         <v>9</v>
@@ -1077,56 +1081,56 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>19-ResumeMuhammadWaqas3y.pdf</t>
+          <t>18-ResumeMuhammadTahaYasin.pdf</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Resumemuhammadwaqas3Y</t>
+          <t>About Me</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mwbkkj@gmail.com</t>
+          <t>mtahayasin07@gmail.com</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>03126318724</t>
+          <t>03406991719</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>github, javascript, state management, html, react, redux, css, react.js</t>
+          <t>html, chrome devtools, react, problem solving, react.js, figma, vs code, css, git, bootstrap, vite, tailwind css, github, javascript, yarn, npm</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>3 years 0 months</t>
+          <t>5 years 6 months</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>3</v>
+        <v>5.5</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>master</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Master of Management Science (Finance-18 year edu) from IMSciences, Hayatabad</t>
+          <t>BS Software Engineering</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via month-name + year-only + year-only + year-only-fuzzy</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>73.45999999999999</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="N11" t="n">
         <v>10</v>
@@ -1135,38 +1139,38 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12-ResumeIjlalSHAH-2y.pdf</t>
+          <t>ResumeHafizAhmad.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Ijlal Shah</t>
+          <t>Hafiz Rehan Ahmad</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ijlalshahzr@gmail.com</t>
+          <t>rehanansari3973@gmail.com</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>+923181669799</t>
+          <t>03099332253</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>javascript, state management, git, bootstrap, redux toolkit, react hooks, context api, html, angular, react, jquery, redux, typescript, lazy loading, css, material ui, react.js</t>
+          <t>responsive design, jwt, react.js, figma, mysql, cypress, agile, react hooks, react, node.js, typescript, lazy loading, tailwind css, ci/cd pipelines, css, redux, authentication, communication, aws, javascript, redux toolkit, teamwork, project management, html, state management, git, jest, mongodb, express</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2 years 0 months</t>
+          <t>2 years 4 months</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1175,16 +1179,16 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Bachelor (inferred) / No major degree found but mentions university</t>
+          <t>I pursued Bachelor of Science in Computer Science (BSc CS) from GC University.</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>72.69</v>
+        <v>76.03</v>
       </c>
       <c r="N12" t="n">
         <v>11</v>
@@ -1193,64 +1197,56 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>27-Hamza Hamid 3y+.pdf</t>
+          <t>19-ResumeMuhammadWaqas3y.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hamza Hamid</t>
+          <t>Resumemuhammadwaqas3Y</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>thedev.hamza@gmail.com</t>
+          <t>Mwbkkj@gmail.com</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>03168767587</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/hamxa-hamid/</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>https://github.com/dadhsahb</t>
-        </is>
-      </c>
+          <t>03126318724</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>github, javascript, chakra ui, tailwind css, git, bootstrap, css, html, react, jquery, vue.js, react.js</t>
+          <t>html, firebase, react, react.js, state management, ios, python, css, redux, android, github, javascript, project management</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1 years 11 months</t>
+          <t>3 years 0 months</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>1.9</v>
+        <v>3</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>master</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Bachelor of Science</t>
+          <t>Master of Management Science (Finance-18 year edu) from IMSciences, Hayatabad</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>date_range via mm/yyyy + year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>70.70999999999999</v>
+        <v>73.45999999999999</v>
       </c>
       <c r="N13" t="n">
         <v>12</v>
@@ -1259,29 +1255,29 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>15-ResumeMuhammadLihaz2y.pdf</t>
+          <t>12-ResumeIjlalSHAH-2y.pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Muhammad Lihaz Ali</t>
+          <t>Ijlal Shah</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>lehazalil23@gmail.com</t>
+          <t>ijlalshahzr@gmail.com</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>03488899315</t>
+          <t>+923181669799</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>javascript, tailwind css, next.js, responsive design, html, typescript, react, css, material ui, react.js</t>
+          <t>react.js, asp.net, agile, sql, react hooks, react, typescript, lazy loading, angular, monitoring, jquery, .net, authorization, context api, css, redux, authentication, communication, javascript, redux toolkit, html, state management, material ui, git, bootstrap, mongodb</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1299,7 +1295,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>BS Software Engineering Jan 2020 - Feb 2024</t>
+          <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1308,7 +1304,7 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>69.62</v>
+        <v>72.69</v>
       </c>
       <c r="N14" t="n">
         <v>13</v>
@@ -1317,46 +1313,46 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>10-ResumeAQIBZAIB-2y.pdf</t>
+          <t>27-Hamza Hamid 3y+.pdf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Aqib Zaib</t>
+          <t>Hamza Hamid</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>chaqib4u@gmail.com</t>
+          <t>thedev.hamza@gmail.com</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>+923040505345</t>
+          <t>03168767587</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/aqib-zaib-</t>
+          <t>https://www.linkedin.com/in/hamxa-hamid/</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://github.com/aqibzaib</t>
+          <t>https://github.com/dadhsahb</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>github, javascript, tailwind css, git, css, redux toolkit, next.js, react query, react, vercel, redux, vue.js, figma, react.js</t>
+          <t>postgresql, vue.js, react.js, docker, asp.net, gcp, sql, react, node.js, chakra ui, azure, tailwind css, github, jquery, .net, java, css, aws, javascript, html, git, bootstrap, s3, mongodb, express</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1 years 6 months</t>
+          <t>1 years 11 months</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1365,7 +1361,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>BS SOFTWARE</t>
+          <t>Bachelor of Science</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1374,7 +1370,7 @@
         </is>
       </c>
       <c r="M15" t="n">
-        <v>66.54000000000001</v>
+        <v>70.70999999999999</v>
       </c>
       <c r="N15" t="n">
         <v>14</v>
@@ -1383,47 +1379,47 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shubham_Mishra_Resume_09-08-2022-16-16-14.pdf</t>
+          <t>15-ResumeMuhammadLihaz2y.pdf</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Shubham Mishra</t>
+          <t>Muhammad Lihaz Ali</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>shubham.mishra@gmail.com</t>
+          <t>lehazalil23@gmail.com</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>9876543210</t>
+          <t>03488899315</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>github, javascript, git, bootstrap, bitbucket, rest api</t>
+          <t>html, next.js, react, responsive design, react.js, typescript, node.js, material ui, css, tailwind css, javascript, mongodb, express</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>3 years 0 months</t>
+          <t>2 years 0 months</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>master</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Master of Computer Applications</t>
+          <t>BS Software Engineering Jan 2020 - Feb 2024</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1432,7 +1428,7 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>64.23</v>
+        <v>69.62</v>
       </c>
       <c r="N16" t="n">
         <v>15</v>
@@ -1441,56 +1437,64 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Rahul_Mishra_Resume_09-08-2022-16-00-15.pdf</t>
+          <t>10-ResumeAQIBZAIB-2y.pdf</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Rahul Mishra</t>
+          <t>Aqib Zaib</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>rahul.mishra@gmail.com</t>
+          <t>chaqib4u@gmail.com</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>9876543210</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+          <t>+923040505345</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/aqib-zaib-</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://github.com/aqibzaib</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>github, javascript, git, bootstrap, bitbucket, rest api</t>
+          <t>next.js, vue.js, react, react.js, figma, css, redux, git, tailwind css, github, react query, javascript, redux toolkit, vercel</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>4 years 0 months</t>
+          <t>1 years 6 months</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>master</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Master of Computer Applications, National Institute of Technology Allahabad (MNNIT), U.P</t>
+          <t>BS SOFTWARE</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via mm/yyyy + year-only</t>
         </is>
       </c>
       <c r="M17" t="n">
-        <v>64.23</v>
+        <v>66.54000000000001</v>
       </c>
       <c r="N17" t="n">
         <v>16</v>
@@ -1499,33 +1503,29 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>17-ResumeMuhammadShayan3y.pdf</t>
+          <t>Shubham_Mishra_Resume_09-08-2022-16-16-14.pdf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Muhammad Shayan</t>
+          <t>Shubham Mishra</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>kshayan091@gmail.com</t>
+          <t>shubham.mishra@gmail.com</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>+923168104861</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/shayan-khan20</t>
-        </is>
-      </c>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>github, javascript, next.js, typescript, react, redux, material ui, figma, seo optimization</t>
+          <t>kubernetes, python, bitbucket, mysql, docker, hive, flask, kafka, redshift, sql, azure, github, monitoring, cloudwatch, java, cassandra, aws, javascript, spark, bigquery, hadoop, git, bootstrap, s3, django, grafana, rest api, linux</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>high school</t>
+          <t>master</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Higher school January 2020– March 2022</t>
+          <t>Master of Computer Applications</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1552,7 +1552,7 @@
         </is>
       </c>
       <c r="M18" t="n">
-        <v>63.38</v>
+        <v>64.23</v>
       </c>
       <c r="N18" t="n">
         <v>17</v>
@@ -1561,51 +1561,47 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11-ResumeEJAZAHMAD.pdf</t>
+          <t>Rahul_Mishra_Resume_09-08-2022-16-00-15.pdf</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Ejaz Ahmad</t>
+          <t>Rahul Mishra</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ayanejaz420fwisg_dpy@indeedemail.com</t>
+          <t>rahul.mishra@gmail.com</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>+923313322420</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/in/ejaz-ahmad-2359a2247</t>
-        </is>
-      </c>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>html, typescript, react, css, rest api, less, graphql</t>
+          <t>kubernetes, python, bitbucket, mysql, docker, hive, flask, kafka, redshift, sql, azure, github, monitoring, cloudwatch, java, cassandra, aws, javascript, spark, bigquery, hadoop, git, bootstrap, s3, django, grafana, rest api, linux</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2 years 0 months</t>
+          <t>4 years 0 months</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>master</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Bachelor (inferred) / No major degree found but mentions university</t>
+          <t>Master of Computer Applications, National Institute of Technology Allahabad (MNNIT), U.P</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1614,7 +1610,7 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>63.38</v>
+        <v>64.23</v>
       </c>
       <c r="N19" t="n">
         <v>18</v>
@@ -1623,46 +1619,42 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>7-Muhammad Yasin - Software Engineer.pdf</t>
+          <t>11-ResumeEJAZAHMAD.pdf</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Muhammad Yasin Software Engineer</t>
+          <t>Ejaz Ahmad</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>yasinwaheed11@gmail.com</t>
+          <t>ayanejaz420fwisg_dpy@indeedemail.com</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>+923026770777</t>
+          <t>+923313322420</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/yasinwahid111</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>https://github.com/YasinWahid</t>
-        </is>
-      </c>
+          <t>https://linkedin.com/in/ejaz-ahmad-2359a2247</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>github, javascript, git, bootstrap, responsive design, html, angular, react, typescript, css, figma, react.js</t>
+          <t>html, react, graphql, mongodb, typescript, css, less, rest api</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1 years 2 months</t>
+          <t>2 years 0 months</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1671,16 +1663,16 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Hifah Technologies | Abbottabad Bachelor of Software Engineering</t>
+          <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M20" t="n">
-        <v>63.21</v>
+        <v>63.38</v>
       </c>
       <c r="N20" t="n">
         <v>19</v>
@@ -1689,64 +1681,60 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Data_engineer(Sample 4+ year).pdf</t>
+          <t>17-ResumeMuhammadShayan3y.pdf</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Biswajit Khetan</t>
+          <t>Muhammad Shayan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>bisjwa1445@gmail.com</t>
+          <t>kshayan091@gmail.com</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>+91987654321</t>
+          <t>+923168104861</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/11i/</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>https://github.com/AnkitDB9</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/in/shayan-khan20</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>github, rest api</t>
+          <t>oauth, jwt, figma, ruby, firebase, react, node.js, typescript, github, redux, authentication, rails, javascript, aws, seo optimization, next.js, react native, material ui, mongodb, express</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>4 years 8 months</t>
+          <t>3 years 0 months</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>4.7</v>
+        <v>3</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>high school</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Bachelor of Technology,</t>
+          <t>Higher school January 2020– March 2022</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only-fuzzy</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M21" t="n">
-        <v>63.08</v>
+        <v>63.38</v>
       </c>
       <c r="N21" t="n">
         <v>20</v>
@@ -1755,64 +1743,64 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>resume_juanjosecarin.pdf</t>
+          <t>7-Muhammad Yasin - Software Engineer.pdf</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Juan Jose Carin</t>
+          <t>Muhammad Yasin Software Engineer</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>juanjose.carin@gmail.com</t>
+          <t>yasinwaheed11@gmail.com</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>940416503364590</t>
+          <t>+923026770777</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://linkedin.com/in/juanjosecarin</t>
+          <t>https://www.linkedin.com/in/yasinwahid111</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://github.com/juanjocarin/W261-Machine-Learning-At-Scale/blob/master/Week07-MrJob/MIDS-W261-2015-HWK-Week07-CarinLlopSatpati-groupZ.ipynb</t>
+          <t>https://github.com/YasinWahid</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>github, git</t>
+          <t>html, react native, firebase, react.js, figma, react, typescript, responsive design, css, git, bootstrap, communication, github, angular, javascript</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>5 years 1 months</t>
+          <t>1 years 2 months</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>5.1</v>
+        <v>1.2</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>master</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Master of Information and Data Science</t>
+          <t>Hifah Technologies | Abbottabad Bachelor of Software Engineering</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only-fuzzy</t>
+          <t>date_range via fuzzy-month + month-name + year-only</t>
         </is>
       </c>
       <c r="M22" t="n">
-        <v>63.08</v>
+        <v>63.21</v>
       </c>
       <c r="N22" t="n">
         <v>21</v>
@@ -1821,56 +1809,64 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>24-ResumeTayyabHussainshah.pdf</t>
+          <t>resume_juanjosecarin.pdf</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tayyab Hussain Shah</t>
+          <t>Juan Jose Carin</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>tayabsajid5@gmail.com</t>
+          <t>juanjose.carin@gmail.com</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>+923365298230</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
+          <t>940416503364590</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/juanjosecarin</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://github.com/juanjocarin/W261-Machine-Learning-At-Scale/blob/master/Week07-MrJob/MIDS-W261-2015-HWK-Week07-CarinLlopSatpati-groupZ.ipynb</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>github, javascript, tailwind css, git, vite, next.js, angular, react, sass, redux, vercel, typescript, css, figma, react.js</t>
+          <t>matplotlib, scikit-learn, python, mysql, hive, statistics, sql, r, github, monitoring, machine learning, communication, aws, spark, ec2, hadoop, git, data visualization, s3, tensorflow, sqlite</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1 years 4 months</t>
+          <t>5 years 1 months</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>1.3</v>
+        <v>5.1</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>master</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Bachelor of Science in Software Engineering</t>
+          <t>Master of Information and Data Science</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only-fuzzy</t>
         </is>
       </c>
       <c r="M23" t="n">
-        <v>62.95</v>
+        <v>63.08</v>
       </c>
       <c r="N23" t="n">
         <v>22</v>
@@ -1879,46 +1875,46 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>22-ResumeSaadAhmad-1y.pdf</t>
+          <t>Data_engineer(Sample 4+ year).pdf</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Saad Ahmad</t>
+          <t>Biswajit Khetan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>saadahmad6830879@gmail.com</t>
+          <t>bisjwa1445@gmail.com</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>923176830879</t>
+          <t>+91987654321</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://linkedin.com/in/saadahmad879</t>
+          <t>https://www.linkedin.com/in/11i/</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://github.com/SaADii09</t>
+          <t>https://github.com/AnkitDB9</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>github, javascript, state management, tailwind css, git, html, react, redux, css, react.js</t>
+          <t>postgresql, kubernetes, python, mysql, nosql, hive, flask, agile, sql, mongodb, azure, github, monitoring, java, cassandra, machine learning, aws, spark, problem solving, ec2, hadoop, s3, rest api, docker</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>0 years 8 months</t>
+          <t>4 years 8 months</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>0.7</v>
+        <v>4.7</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1927,16 +1923,16 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>BS Computer Science</t>
+          <t>Bachelor of Technology,</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only-fuzzy</t>
         </is>
       </c>
       <c r="M24" t="n">
-        <v>61.28</v>
+        <v>63.08</v>
       </c>
       <c r="N24" t="n">
         <v>23</v>
@@ -1945,38 +1941,38 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Shubham_Mishra_Resume_10-08-2022-16-06-13.pdf</t>
+          <t>24-ResumeTayyabHussainshah.pdf</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Shubham Mishra</t>
+          <t>Tayyab Hussain Shah</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>shubham.mishra@gmail.com</t>
+          <t>tayabsajid5@gmail.com</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>9876543210</t>
+          <t>+923365298230</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>github, git, jenkins, bitbucket, rest api</t>
+          <t>postgresql, react.js, figma, python, php, mysql, nosql, agile, sql, firebase, react, node.js, typescript, vite, tailwind css, github, angular, vercel, css, redux, laravel, javascript, project management, flutter, next.js, sass, git, django, mongodb, express</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>7 years 0 months</t>
+          <t>1 years 4 months</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>7</v>
+        <v>1.3</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -1985,16 +1981,16 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Bachelor of Engineering in Computer Science,</t>
+          <t>Bachelor of Science in Software Engineering</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
       <c r="M25" t="n">
-        <v>61.15</v>
+        <v>62.95</v>
       </c>
       <c r="N25" t="n">
         <v>24</v>
@@ -2003,64 +1999,64 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1-Fahadalamresume.pdf</t>
+          <t>22-ResumeSaadAhmad-1y.pdf</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Fahad Alam</t>
+          <t>Saad Ahmad</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>fahadalam12405@gmail.com</t>
+          <t>saadahmad6830879@gmail.com</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>+923272748498</t>
+          <t>923176830879</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/fahad-alam</t>
+          <t>https://linkedin.com/in/saadahmad879</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://github.com/Fahad12405</t>
+          <t>https://github.com/SaADii09</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>state management, bootstrap, redux toolkit, context api, react, webpack, javascript, postcss, git, next.js, html, jquery, css, vite, redux, vue.js, github, tailwind css, axios, typescript, react.js</t>
+          <t>jwt, react.js, python, sql, firebase, react, node.js, r, tailwind css, github, authorization, css, redux, authentication, javascript, flutter, html, state management, git, mongodb, express</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1 years 3 months</t>
+          <t>0 years 8 months</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>high school</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Intermediate, Cs</t>
+          <t>BS Computer Science</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>date_range via reverse-order</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
       <c r="M26" t="n">
-        <v>60.19</v>
+        <v>61.28</v>
       </c>
       <c r="N26" t="n">
         <v>25</v>
@@ -2069,42 +2065,38 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Nezuko_Kamado_Resume_10-08-2022-16-04-20.pdf</t>
+          <t>Shubham_Mishra_Resume_10-08-2022-16-06-13.pdf</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Kamado Associate Lead</t>
+          <t>Shubham Mishra</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>hello.ineuron@gmail.com</t>
+          <t>shubham.mishra@gmail.com</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>9923312341</t>
+          <t>9876543210</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>https://github.com/model</t>
-        </is>
-      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>github, rest api</t>
+          <t>jenkins, kubernetes, python, bitbucket, mysql, docker, hive, kafka, redshift, sql, azure, github, monitoring, cloudwatch, java, cassandra, authentication, aws, spark, bigquery, hadoop, git, grafana, s3, rest api, linux</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>6 years 0 months</t>
+          <t>7 years 0 months</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -2113,7 +2105,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Bachelor Of Technology in Computer Science</t>
+          <t>Bachelor of Engineering in Computer Science,</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2122,7 +2114,7 @@
         </is>
       </c>
       <c r="M27" t="n">
-        <v>60.08</v>
+        <v>61.15</v>
       </c>
       <c r="N27" t="n">
         <v>26</v>
@@ -2131,46 +2123,46 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2-TouseefAbidCv.pdf</t>
+          <t>1-Fahadalamresume.pdf</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Touseef Abid</t>
+          <t>Fahad Alam</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>touseefabid737@gmail.com</t>
+          <t>fahadalam12405@gmail.com</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>+923102939875</t>
+          <t>+923272748498</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/touseefabid</t>
+          <t>https://www.linkedin.com/in/fahad-alam</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://github.com/Touseef4705</t>
+          <t>https://github.com/Fahad12405</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>github, javascript, git, npm, redux toolkit, next.js, yarn, html, react, vercel, redux, css, react.js, react router</t>
+          <t>vue.js, react.js, firebase, react, node.js, typescript, vite, tailwind css, github, jquery, webpack, context api, css, redux, postcss, javascript, redux toolkit, html, axios, next.js, state management, git, bootstrap, mongodb, express</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1 years 6 months</t>
+          <t>1 years 3 months</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -2179,16 +2171,16 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Intermediate, Business Commerce</t>
+          <t>Intermediate, Cs</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
+          <t>date_range via reverse-order</t>
         </is>
       </c>
       <c r="M28" t="n">
-        <v>59.62</v>
+        <v>60.19</v>
       </c>
       <c r="N28" t="n">
         <v>27</v>
@@ -2197,46 +2189,42 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>16-ResumeMuhammadluqmanKhan1y+.pdf</t>
+          <t>Nezuko_Kamado_Resume_10-08-2022-16-04-20.pdf</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Muhammad Luqman</t>
+          <t>Kamado Associate Lead</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>IK3281751@gmail.com</t>
+          <t>hello.ineuron@gmail.com</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>+923361935561</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>https://linkedin.com/in/muhammad-luqman-khan-051047267</t>
-        </is>
-      </c>
+          <t>9923312341</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://github.com/Luqmanoffical</t>
+          <t>https://github.com/model</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>github, javascript, bootstrap, html, typescript, react, css, figma, react.js, netlify</t>
+          <t>matplotlib, kubernetes, python, flask, statistics, kafka, gcp, linear regression, pandas, deep learning, azure, probability, github, numpy, seaborn, prometheus, clustering, machine learning, dimensionality, aws, grpc, fastapi, django, grafana, tensorflow, pytorch, rest api, keras, docker</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1 years 0 months</t>
+          <t>6 years 0 months</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -2245,16 +2233,16 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Bachelor's Degree in Information Technology</t>
+          <t>Bachelor Of Technology in Computer Science</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>date_range via year-only + year-only-fuzzy</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M29" t="n">
-        <v>58.46</v>
+        <v>60.08</v>
       </c>
       <c r="N29" t="n">
         <v>28</v>
@@ -2263,37 +2251,37 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ScholarCV.pdf</t>
+          <t>2-TouseefAbidCv.pdf</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Muhammad Aqeel</t>
+          <t>Touseef Abid</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>maqeelcs09@gmail.com</t>
+          <t>touseefabid737@gmail.com</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>+923419905547</t>
+          <t>+923102939875</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://linkedin.com/in/aqeelkhan09</t>
+          <t>https://www.linkedin.com/in/touseefabid</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://github.com/maqeel019</t>
+          <t>https://github.com/Touseef4705</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>github, javascript, git, html, css</t>
+          <t>yarn, html, next.js, react, firebase, react.js, css, redux, git, authentication, react router, github, javascript, redux toolkit, npm, vercel</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2306,12 +2294,12 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>high school</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Bachelor of Computer Science</t>
+          <t>Intermediate, Business Commerce</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -2320,7 +2308,7 @@
         </is>
       </c>
       <c r="M30" t="n">
-        <v>57.31</v>
+        <v>59.62</v>
       </c>
       <c r="N30" t="n">
         <v>29</v>
@@ -2329,46 +2317,46 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MAqeel.pdf</t>
+          <t>16-ResumeMuhammadluqmanKhan1y+.pdf</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Muhammad Aqeel</t>
+          <t>Muhammad Luqman</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>maqeelcs09@gmail.com</t>
+          <t>IK3281751@gmail.com</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>+923419905547</t>
+          <t>+923361935561</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://linkedin.com/in/aqeelkhan09</t>
+          <t>https://linkedin.com/in/muhammad-luqman-khan-051047267</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://github.com/maqeel019</t>
+          <t>https://github.com/Luqmanoffical</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>github, javascript, git, html, css</t>
+          <t>html, react, node.js, react.js, figma, typescript, css, bootstrap, netlify, nosql, github, javascript, mongodb, express, sql</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1 years 6 months</t>
+          <t>1 years 0 months</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -2377,16 +2365,16 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Bachelor of Computer Science</t>
+          <t>Bachelor's Degree in Information Technology</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
+          <t>date_range via year-only + year-only-fuzzy</t>
         </is>
       </c>
       <c r="M31" t="n">
-        <v>57.31</v>
+        <v>58.46</v>
       </c>
       <c r="N31" t="n">
         <v>30</v>
@@ -2395,42 +2383,46 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Naruto_uzumaki_Resume_10-08-2022-15-31-44.pdf</t>
+          <t>ScholarCV.pdf</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Naruto Uzumaki</t>
+          <t>Muhammad Aqeel</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>hello.ineuron@gmail.com</t>
+          <t>maqeelcs09@gmail.com</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>9923312341</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
+          <t>+923419905547</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/aqeelkhan09</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://github.com/PROFILE</t>
+          <t>https://github.com/maqeel019</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>github</t>
+          <t>matplotlib, streamlit, python, mysql, load balancing, sql, pandas, github, vs code, numpy, seaborn,  hypothesis testing, css, machine learning, communication, jupyter, javascript, project management, html, critical thinking, git, decision trees, jupyter notebook</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>4 years 0 months</t>
+          <t>1 years 6 months</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -2439,16 +2431,16 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Bachelor Of Technology in Computer Science, Jaypee Institute Of Information Technology</t>
+          <t>Bachelor of Computer Science</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
       <c r="M32" t="n">
-        <v>57</v>
+        <v>57.31</v>
       </c>
       <c r="N32" t="n">
         <v>31</v>
@@ -2457,42 +2449,46 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>3-AJSwatiResume.pdf</t>
+          <t>MAqeel.pdf</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Abdullah Javed</t>
+          <t>Muhammad Aqeel</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>abdullah.javed9438@gmail.com</t>
+          <t>maqeelcs09@gmail.com</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>+923499377144</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
+          <t>+923419905547</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/aqeelkhan09</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://github.com/AbdullahKhanSwati</t>
+          <t>https://github.com/maqeel019</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>github, javascript, state management, tailwind css, react hooks, responsive design, react, jquery, redux, lazy loading, css, react.js, netlify</t>
+          <t>matplotlib, streamlit, python, mysql, load balancing, plotly, sql, linear regression, pandas, probability, github, vs code, numpy, seaborn, clustering,  hypothesis testing, css, dimensionality, machine learning, communication, jupyter, cross-validation, javascript, project management, supervised, html, feature engineering, etl pipelines, unsupervised learning, hyperparameter tuning, git, decision trees, jupyter notebook, linux</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1 years 0 months</t>
+          <t>1 years 6 months</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -2501,16 +2497,16 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Bachelor (inferred) / No major degree found but mentions university</t>
+          <t>Bachelor of Computer Science</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>date_range via year-only-fuzzy</t>
+          <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
       <c r="M33" t="n">
-        <v>55.46</v>
+        <v>57.31</v>
       </c>
       <c r="N33" t="n">
         <v>32</v>
@@ -2519,17 +2515,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Tanjiro_Bhatia_Resume_09-08-2022-19-15-13.pdf</t>
+          <t>Naruto_uzumaki_Resume_10-08-2022-15-31-44.pdf</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Tanjiro Bhatia</t>
+          <t>Naruto Uzumaki</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Tanjiro.bhatia67@gmail.com</t>
+          <t>hello.ineuron@gmail.com</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2538,15 +2534,23 @@
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://github.com/PROFILE</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>clustering, deep learning,  hypothesis testing, azure, python, machine learning, probability, kafka, jupyter notebook, jupyter, github, aws, statistics, spark, docker</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>6 years 0 months</t>
+          <t>4 years 0 months</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -2555,7 +2559,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Bachelor (inferred) / No major degree found but mentions university</t>
+          <t>Bachelor Of Technology in Computer Science, Jaypee Institute Of Information Technology</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -2564,7 +2568,7 @@
         </is>
       </c>
       <c r="M34" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="N34" t="n">
         <v>33</v>
@@ -2573,42 +2577,42 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>21-ResumeRehmanZeb2y+.pdf</t>
+          <t>3-AJSwatiResume.pdf</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Resumerehmanzeb2Y+</t>
+          <t>Abdullah Javed</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>rehmanzeb2k17@gmail.com</t>
+          <t>abdullah.javed9438@gmail.com</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>+923119449029</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/rehmanzeb</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
+          <t>+923499377144</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://github.com/AbdullahKhanSwati</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>javascript, tailwind css, git, bootstrap, next.js, responsive design, react, css, react.js</t>
+          <t>responsive design, jwt, react.js, nosql, sql, react hooks, firebase, react, node.js, lazy loading, netlify, tailwind css, github, jquery, java, css, redux, authentication, android, aws, javascript, react native, state management, kotlin, mongodb, express</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>0 years 9 months</t>
+          <t>1 years 0 months</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
@@ -2617,16 +2621,16 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>BS Computer Science</t>
+          <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only + month-only + year</t>
+          <t>date_range via year-only-fuzzy</t>
         </is>
       </c>
       <c r="M35" t="n">
-        <v>53.96</v>
+        <v>55.46</v>
       </c>
       <c r="N35" t="n">
         <v>34</v>
@@ -2635,30 +2639,46 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>data-scientist-resume-sample-template.pdf</t>
+          <t>ResumeIbrahimAhmed.pdf</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Robin Doe</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
+          <t>Ibrahim Ahmed</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ibrahimahmed12333@gmail.com</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>123451234567090</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
+          <t>+923431938944</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ibrahim-ahmed-8b8961254</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://github.com/IbrahimAhmed413</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>html, java, react, node.js, react.js, material ui, css, communication, github, mongodb, express</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>8 years 6 months</t>
+          <t>1 years 0 months</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>8.5</v>
+        <v>1</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -2667,16 +2687,16 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>ba Eng al) - AMT</t>
+          <t>Bachelor of Computer Science</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>date_range via year-only + year-only-fuzzy</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M36" t="n">
-        <v>52</v>
+        <v>55.38</v>
       </c>
       <c r="N36" t="n">
         <v>35</v>
@@ -2685,38 +2705,38 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>20-ResumeRAJAABDULLAH1.5y.pdf</t>
+          <t>Tanjiro_Bhatia_Resume_09-08-2022-19-15-13.pdf</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Raja Abdullah</t>
+          <t>Tanjiro Bhatia</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>rabdullah806@gmail.com</t>
+          <t>Tanjiro.bhatia67@gmail.com</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>923175510676</t>
+          <t>9923312341</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>html, javascript, css</t>
+          <t>deep learning, azure, python, machine learning, kafka, aws, spark, docker</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1 years 6 months</t>
+          <t>6 years 0 months</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>1.5</v>
+        <v>6</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -2734,7 +2754,7 @@
         </is>
       </c>
       <c r="M37" t="n">
-        <v>49.23</v>
+        <v>55</v>
       </c>
       <c r="N37" t="n">
         <v>36</v>
@@ -2743,42 +2763,42 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Nitish Kumar.pdf</t>
+          <t>21-ResumeRehmanZeb2y+.pdf</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Nitish Kumar</t>
+          <t>Resumerehmanzeb2Y+</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>xyz@gmail.com</t>
+          <t>rehmanzeb2k17@gmail.com</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>9977141714</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>https://github.com/vishalsingh17</t>
-        </is>
-      </c>
+          <t>+923119449029</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/rehmanzeb</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>html, css, git, github</t>
+          <t>next.js, react, problem solving, react.js, responsive design, css, git, bootstrap, communication, tailwind css, r, javascript</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1 years 0 months</t>
+          <t>0 years 9 months</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -2787,16 +2807,16 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>12/2015 – 12/2018 BCA</t>
+          <t>BS Computer Science</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via fuzzy-month + month-name + year-only + month-only + year</t>
         </is>
       </c>
       <c r="M38" t="n">
-        <v>46.23</v>
+        <v>53.96</v>
       </c>
       <c r="N38" t="n">
         <v>37</v>
@@ -2805,64 +2825,52 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5-JAWADRESUME.pdf</t>
+          <t>data-scientist-resume-sample-template.pdf</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Jawad Ali</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>jawadalikhan359@gmail.com</t>
-        </is>
-      </c>
+          <t>Robin Doe</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>03139908709</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/jawadali1535</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>https://github.com/JawadAli1535</t>
-        </is>
-      </c>
+          <t>123451234567090</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>github, javascript, tailwind css, git, axios, sass, react, vercel, redux, jquery, typescript, css</t>
+          <t>machine learning</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>0 years 5 months</t>
+          <t>8 years 6 months</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>0.4</v>
+        <v>8.5</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>high school</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Nodejs(intermediate)</t>
+          <t>ba Eng al) - AMT</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only</t>
+          <t>date_range via year-only + year-only-fuzzy</t>
         </is>
       </c>
       <c r="M39" t="n">
-        <v>45.71</v>
+        <v>52</v>
       </c>
       <c r="N39" t="n">
         <v>38</v>
@@ -2871,34 +2879,38 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Riya_Bhatiya_Resume_09-08-2022-19-26-53.pdf</t>
+          <t>20-ResumeRAJAABDULLAH1.5y.pdf</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Riya Bhatiya</t>
+          <t>Raja Abdullah</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>riya.bhatia67@gmail.com</t>
+          <t>rabdullah806@gmail.com</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>9923312341</t>
+          <t>923175510676</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>html, .net, css, communication, monitoring, asp.net, agile, javascript, project management, sql</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>2 years 0 months</t>
+          <t>1 years 6 months</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -2907,7 +2919,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Bachelor Of Technology in Computer Science Freelance Mentor Of Data Structure and Algorithms</t>
+          <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -2916,7 +2928,7 @@
         </is>
       </c>
       <c r="M40" t="n">
-        <v>45</v>
+        <v>49.23</v>
       </c>
       <c r="N40" t="n">
         <v>39</v>
@@ -2925,51 +2937,51 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Shankar_chavan_Resume_10-08-2022-12-54-00.pdf</t>
+          <t>Nitish Kumar.pdf</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Shankar Chavan</t>
+          <t>Nitish Kumar</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>shankar.chavan@gmail.com</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/</t>
-        </is>
-      </c>
+          <t>xyz@gmail.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>9977141714</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://github.com/</t>
+          <t>https://github.com/vishalsingh17</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>github</t>
+          <t>matplotlib, streamlit, python, mysql, plotly, flask, sql, pandas, deep learning, github, numpy, css, machine learning, aws, html, feature engineering, ec2, express, git, django, redis, mongodb, docker</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1 years 6 months</t>
+          <t>1 years 0 months</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>master</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Master Degree, SPPU University</t>
+          <t>12/2015 – 12/2018 BCA</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -2978,7 +2990,7 @@
         </is>
       </c>
       <c r="M41" t="n">
-        <v>43</v>
+        <v>46.23</v>
       </c>
       <c r="N41" t="n">
         <v>40</v>
@@ -2987,60 +2999,64 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>26-Sameer Khan Cv3y.pdf</t>
+          <t>5-JAWADRESUME.pdf</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Sameer Khan</t>
+          <t>Jawad Ali</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>berlanjan123@gmail.com</t>
+          <t>jawadalikhan359@gmail.com</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>+923169769253</t>
+          <t>03139908709</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/sameer-khan-660966251</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
+          <t>https://www.linkedin.com/in/jawadali1535</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://github.com/JawadAli1535</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>github, bootstrap, next.js, html, react, css</t>
+          <t>axios, react, mongodb, typescript, php, css, redux, mysql, sass, git, tailwind css, github, javascript, jquery, vercel, sql</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>0 years 0 months</t>
+          <t>0 years 5 months</t>
         </is>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>high school</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Degree Bs Computer Science</t>
+          <t>Nodejs(intermediate)</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>none via none</t>
+          <t>date_range via fuzzy-month + month-name + year-only</t>
         </is>
       </c>
       <c r="M42" t="n">
-        <v>37.23</v>
+        <v>45.71</v>
       </c>
       <c r="N42" t="n">
         <v>41</v>
@@ -3049,38 +3065,38 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>8-Raja Muhammad Awais.pdf</t>
+          <t>Riya_Bhatiya_Resume_09-08-2022-19-26-53.pdf</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Raja Muhammad Awais</t>
+          <t>Riya Bhatiya</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>muhammadawaisturk1@gmail.com</t>
+          <t>riya.bhatia67@gmail.com</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>+923155406093</t>
+          <t>9923312341</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>gitlab, git</t>
+          <t>deep learning,  hypothesis testing, azure, python, machine learning, probability, kafka, aws, statistics, spark, docker</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>0 years 0 months</t>
+          <t>2 years 0 months</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -3089,16 +3105,16 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>BS COMPUTER SCIENCE Abbottabad University Of Science And Technology</t>
+          <t>Bachelor Of Technology in Computer Science Freelance Mentor Of Data Structure and Algorithms</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>none via none</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M43" t="n">
-        <v>28.08</v>
+        <v>45</v>
       </c>
       <c r="N43" t="n">
         <v>42</v>
@@ -3107,55 +3123,241 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Muhammad Abu Aqeel Europass.pdf</t>
+          <t>Shankar_chavan_Resume_10-08-2022-12-54-00.pdf</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Muhammad Abu Aqeel</t>
+          <t>Shankar Chavan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>maqeelcs09@gmail.com</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>+923419905547</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
+          <t>shankar.chavan@gmail.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://github.com/</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>linear regression, problem solving, kubernetes, deep learning, cassandra, python, machine learning, mysql, tensorflow, github, pytorch, aws, mongodb, docker</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>0 years 0 months</t>
+          <t>1 years 6 months</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>master</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>muhammad abu aqeel nationality: pakistani gender: male phone number: (+92) 3419905547 (mobile) email address: maqeelcs09@gmail.com address: pakistan (home) about me a dedicated individual with a proven track record of achieving and exceeding goals through unwavering determination and a commitment to excellence education and training lahore, pakistan bachelor of science university of swabi field of studycomputer science 2020 bam khel,swabi, pakistan intermediate the glorious college of science &amp; technology language skills mother tongue(s): urdu | pashto other language(s): understanding speaking writing spoken spoken listening reading production interaction english c1 c1 c1 c1 c1 levels: a1 and a2: basic user; b1 and b2: independent user; c1 and c2: proficient user additional information management and leadership skills skills strategic planning and execution: • proficient in developing long-term strategies and effectively executing action plans to achieve organizational goals. • skilled at aligning business objectives with actionable plans for efficient resource utilization. team leadership and motivation: • proven ability to lead and inspire teams, fostering a collaborative and high-performing work environment. • experienced in setting clear expectations, providing constructive feedback, and empowering team members to reach their potential. decision making and problem-solving: • strong analytical and critical thinking skills, enabling effective decision-making in complex situations.</t>
+          <t>Master Degree, SPPU University</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>none via none</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M44" t="n">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="N44" t="n">
         <v>43</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>26-Sameer Khan Cv3y.pdf</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Sameer Khan</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>berlanjan123@gmail.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>+923169769253</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sameer-khan-660966251</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>html, next.js, react, css, bootstrap, github</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>0 years 0 months</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>bachelor</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Degree Bs Computer Science</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>none via none</t>
+        </is>
+      </c>
+      <c r="M45" t="n">
+        <v>37.23</v>
+      </c>
+      <c r="N45" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>8-Raja Muhammad Awais.pdf</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Raja Muhammad Awais</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>muhammadawaisturk1@gmail.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>+923155406093</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>prometheus, firewalls, siem, network security, python, machine learning, git, data visualization, gitlab, monitoring, gitlab ci, aws, linux</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>0 years 0 months</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>bachelor</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>BS COMPUTER SCIENCE Abbottabad University Of Science And Technology</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>none via none</t>
+        </is>
+      </c>
+      <c r="M46" t="n">
+        <v>28.08</v>
+      </c>
+      <c r="N46" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Muhammad Abu Aqeel Europass.pdf</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Muhammad Abu Aqeel</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>maqeelcs09@gmail.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>+923419905547</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>communication, critical thinking</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>0 years 0 months</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>bachelor</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>muhammad abu aqeel nationality: pakistani gender: male phone number: (+92) 3419905547 (mobile) email address: maqeelcs09@gmail.com address: pakistan (home) about me a dedicated individual with a proven track record of achieving and exceeding goals through unwavering determination and a commitment to excellence education and training lahore, pakistan bachelor of science university of swabi field of studycomputer science 2020 bam khel,swabi, pakistan intermediate the glorious college of science &amp; technology language skills mother tongue(s): urdu | pashto other language(s): understanding speaking writing spoken spoken listening reading production interaction english c1 c1 c1 c1 c1 levels: a1 and a2: basic user; b1 and b2: independent user; c1 and c2: proficient user additional information management and leadership skills skills strategic planning and execution: • proficient in developing long-term strategies and effectively executing action plans to achieve organizational goals. • skilled at aligning business objectives with actionable plans for efficient resource utilization. team leadership and motivation: • proven ability to lead and inspire teams, fostering a collaborative and high-performing work environment. • experienced in setting clear expectations, providing constructive feedback, and empowering team members to reach their potential. decision making and problem-solving: • strong analytical and critical thinking skills, enabling effective decision-making in complex situations.</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>none via none</t>
+        </is>
+      </c>
+      <c r="M47" t="n">
+        <v>25</v>
+      </c>
+      <c r="N47" t="n">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
enhance scoring logic, remove redundant parsing, and add progress bar
</commit_message>
<xml_diff>
--- a/output/all_candidates_ranked.xlsx
+++ b/output/all_candidates_ranked.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>eslint, oauth, integration testing, jwt, mysql, hive, agile, react, typescript, nest.js, tailwind css, github, monitoring, spring, spring boot, java, authorization, css, redux, unit testing, authentication, javascript, html, axios, next.js, material ui, git, react query, prettier</t>
+          <t>mysql, react, axios, authentication, hive, typescript, css, nest.js, integration testing, jwt, eslint, material ui, spring boot, github, next.js, java, react query, redux, tailwind css, agile, git, authorization, spring, monitoring, html, javascript, oauth, prettier, unit testing</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>responsive design, react.js, figma, react, node.js, typescript, netlify, tailwind css, github, vs code, vercel, css, redux, authentication, communication, websockets, javascript, redux toolkit, next.js, lighthouse, material ui, git, data visualization, bootstrap, mongodb, express</t>
+          <t>react, authentication, typescript, data visualization, css, figma, redux toolkit, material ui, github, lighthouse, next.js, netlify, vs code, bootstrap, node.js, tailwind css, react.js, responsive design, git, mongodb, javascript, communication, vercel, websockets, express, redux</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>responsive design, react.js, figma, react, node.js, typescript, netlify, tailwind css, github, vs code, vercel, css, redux, authentication, communication, websockets, javascript, redux toolkit, next.js, lighthouse, material ui, git, data visualization, bootstrap, mongodb, express</t>
+          <t>react, authentication, typescript, data visualization, css, figma, redux toolkit, material ui, github, lighthouse, next.js, netlify, vs code, bootstrap, node.js, tailwind css, react.js, responsive design, git, mongodb, javascript, communication, vercel, websockets, express, redux</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>postgresql, vue.js, graphql, responsive design, react.js, figma, cypress, docker, agile, single page applications, react, styled components, node.js, typescript, lazy loading, netlify, tailwind css, github, vercel, github actions, webpack, scrum, css, redux, progressive web apps, aws, seo optimization, javascript, next.js, babel, code splitting, state management, react testing library, git, jest, mongodb, express</t>
+          <t>react, graphql, typescript, css, aws, cypress, figma, vue.js, seo optimization, scrum, github, next.js, netlify, node.js, tailwind css, agile, react.js, code splitting, github actions, responsive design, postgresql, styled components, git, mongodb, react testing library, webpack, javascript, jest, vercel, docker, state management, babel, single page applications, lazy loading, progressive web apps, express, redux</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -793,7 +793,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>graphql, responsive design, react.js, agile, firebase, react, node.js, typescript, azure, tailwind css, css, redux, unit testing, authentication, communication, websockets, aws, javascript, seo optimization, project management, next.js, git, bootstrap, mongodb</t>
+          <t>project management, react, authentication, graphql, typescript, css, aws, seo optimization, next.js, bootstrap, redux, node.js, tailwind css, agile, react.js, azure, responsive design, git, mongodb, javascript, communication, firebase, websockets, unit testing</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>react.js, python, mysql, react hooks, firebase, react, node.js, ios, azure, tailwind css, github, github actions, scrum, css, communication, android, javascript, project management, flutter, material ui, git, mongodb, express</t>
+          <t>mysql, project management, react, css, material ui, scrum, github, python, android, node.js, tailwind css, react.js, github actions, azure, git, mongodb, javascript, communication, react hooks, ios, firebase, flutter, express</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -921,7 +921,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>react.js, figma, mysql, agile, react, node.js, r, tailwind css, authorization, css, redux, laravel, authentication, communication, javascript, html, state management, material ui, git, mongodb, express</t>
+          <t>mysql, react, authentication, css, r, figma, material ui, node.js, tailwind css, laravel, agile, react.js, git, mongodb, authorization, html, javascript, communication, state management, express, redux</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -979,7 +979,7 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>next.js, react, react.js, figma, typescript, material ui, css, git, bootstrap, adobe xd, tailwind css, github, javascript, linux</t>
+          <t>bootstrap, tailwind css, react, figma, react.js, linux, git, material ui, typescript, adobe xd, github, next.js, css, javascript</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>api's integration, firebase, react, azure, machine learning, css, vercel, redux, material ui, docker, tailwind css, github, php, bootstrap, aws, mongodb, express</t>
+          <t>aws, bootstrap, redux, tailwind css, machine learning, vercel, react, firebase, azure, docker, material ui, mongodb, api's integration, github, php, express, css</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1103,7 +1103,7 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>html, chrome devtools, react, problem solving, react.js, figma, vs code, css, git, bootstrap, vite, tailwind css, github, javascript, yarn, npm</t>
+          <t>bootstrap, tailwind css, vite, css, npm, react, figma, react.js, yarn, problem solving, git, chrome devtools, vs code, github, html, javascript</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1161,7 +1161,7 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>responsive design, jwt, react.js, figma, mysql, cypress, agile, react hooks, react, node.js, typescript, lazy loading, tailwind css, ci/cd pipelines, css, redux, authentication, communication, aws, javascript, redux toolkit, teamwork, project management, html, state management, git, jest, mongodb, express</t>
+          <t>mysql, project management, react, authentication, typescript, css, ci/cd pipelines, aws, cypress, figma, jwt, redux toolkit, node.js, tailwind css, agile, react.js, responsive design, git, mongodb, teamwork, html, javascript, communication, jest, react hooks, state management, lazy loading, express, redux</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>76.03</v>
+        <v>75.69</v>
       </c>
       <c r="N12" t="n">
         <v>11</v>
@@ -1219,7 +1219,7 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>html, firebase, react, react.js, state management, ios, python, css, redux, android, github, javascript, project management</t>
+          <t>android, redux, project management, css, react, react.js, ios, firebase, state management, github, python, html, javascript</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1277,7 +1277,7 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>react.js, asp.net, agile, sql, react hooks, react, typescript, lazy loading, angular, monitoring, jquery, .net, authorization, context api, css, redux, authentication, communication, javascript, redux toolkit, html, state management, material ui, git, bootstrap, mongodb</t>
+          <t>react, authentication, typescript, context api, css, redux toolkit, material ui, bootstrap, agile, react.js, git, mongodb, asp.net, authorization, jquery, monitoring, html, javascript, communication, .net, react hooks, sql, state management, lazy loading, angular, redux</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>postgresql, vue.js, react.js, docker, asp.net, gcp, sql, react, node.js, chakra ui, azure, tailwind css, github, jquery, .net, java, css, aws, javascript, html, git, bootstrap, s3, mongodb, express</t>
+          <t>gcp, react, css, aws, vue.js, github, java, bootstrap, node.js, tailwind css, react.js, azure, postgresql, git, mongodb, asp.net, jquery, html, s3, javascript, .net, sql, docker, express, chakra ui</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1370,7 +1370,7 @@
         </is>
       </c>
       <c r="M15" t="n">
-        <v>70.70999999999999</v>
+        <v>70.54000000000001</v>
       </c>
       <c r="N15" t="n">
         <v>14</v>
@@ -1401,7 +1401,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>html, next.js, react, responsive design, react.js, typescript, node.js, material ui, css, tailwind css, javascript, mongodb, express</t>
+          <t>node.js, tailwind css, css, react, react.js, responsive design, material ui, mongodb, typescript, next.js, express, html, javascript</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>next.js, vue.js, react, react.js, figma, css, redux, git, tailwind css, github, react query, javascript, redux toolkit, vercel</t>
+          <t>redux, tailwind css, vercel, react, vue.js, figma, react.js, redux toolkit, git, github, next.js, react query, css, javascript</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1525,7 +1525,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>kubernetes, python, bitbucket, mysql, docker, hive, flask, kafka, redshift, sql, azure, github, monitoring, cloudwatch, java, cassandra, aws, javascript, spark, bigquery, hadoop, git, bootstrap, s3, django, grafana, rest api, linux</t>
+          <t>mysql, bitbucket, kafka, hive, kubernetes, aws, flask, hadoop, github, python, java, bootstrap, azure, git, cloudwatch, monitoring, grafana, s3, rest api, javascript, django, linux, sql, spark, docker, cassandra, bigquery, redshift</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1583,7 +1583,7 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>kubernetes, python, bitbucket, mysql, docker, hive, flask, kafka, redshift, sql, azure, github, monitoring, cloudwatch, java, cassandra, aws, javascript, spark, bigquery, hadoop, git, bootstrap, s3, django, grafana, rest api, linux</t>
+          <t>mysql, bitbucket, kafka, hive, kubernetes, aws, flask, hadoop, github, python, java, bootstrap, azure, git, cloudwatch, monitoring, grafana, s3, rest api, javascript, django, linux, sql, spark, docker, cassandra, bigquery, redshift</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1619,42 +1619,46 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11-ResumeEJAZAHMAD.pdf</t>
+          <t>7-Muhammad Yasin - Software Engineer.pdf</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Ejaz Ahmad</t>
+          <t>Muhammad Yasin Software Engineer</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ayanejaz420fwisg_dpy@indeedemail.com</t>
+          <t>yasinwaheed11@gmail.com</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>+923313322420</t>
+          <t>+923026770777</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://linkedin.com/in/ejaz-ahmad-2359a2247</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
+          <t>https://www.linkedin.com/in/yasinwahid111</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://github.com/YasinWahid</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>html, react, graphql, mongodb, typescript, css, less, rest api</t>
+          <t>bootstrap, communication, css, react, figma, react.js, firebase, responsive design, git, react native, typescript, github, angular, html, javascript</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2 years 0 months</t>
+          <t>1 years 2 months</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1663,16 +1667,16 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Bachelor (inferred) / No major degree found but mentions university</t>
+          <t>Hifah Technologies | Abbottabad Bachelor of Software Engineering</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via fuzzy-month + month-name + year-only</t>
         </is>
       </c>
       <c r="M20" t="n">
-        <v>63.38</v>
+        <v>63.54</v>
       </c>
       <c r="N20" t="n">
         <v>19</v>
@@ -1681,51 +1685,51 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>17-ResumeMuhammadShayan3y.pdf</t>
+          <t>11-ResumeEJAZAHMAD.pdf</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Muhammad Shayan</t>
+          <t>Ejaz Ahmad</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>kshayan091@gmail.com</t>
+          <t>ayanejaz420fwisg_dpy@indeedemail.com</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>+923168104861</t>
+          <t>+923313322420</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/shayan-khan20</t>
+          <t>https://linkedin.com/in/ejaz-ahmad-2359a2247</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>oauth, jwt, figma, ruby, firebase, react, node.js, typescript, github, redux, authentication, rails, javascript, aws, seo optimization, next.js, react native, material ui, mongodb, express</t>
+          <t>css, react, mongodb, less, graphql, typescript, html, rest api</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>3 years 0 months</t>
+          <t>2 years 0 months</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>high school</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Higher school January 2020– March 2022</t>
+          <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1743,64 +1747,60 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>7-Muhammad Yasin - Software Engineer.pdf</t>
+          <t>17-ResumeMuhammadShayan3y.pdf</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Muhammad Yasin Software Engineer</t>
+          <t>Muhammad Shayan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>yasinwaheed11@gmail.com</t>
+          <t>kshayan091@gmail.com</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>+923026770777</t>
+          <t>+923168104861</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/yasinwahid111</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>https://github.com/YasinWahid</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/in/shayan-khan20</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>html, react native, firebase, react.js, figma, react, typescript, responsive design, css, git, bootstrap, communication, github, angular, javascript</t>
+          <t>react, authentication, typescript, aws, figma, jwt, material ui, seo optimization, github, rails, next.js, node.js, mongodb, react native, javascript, ruby, oauth, firebase, express, redux</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1 years 2 months</t>
+          <t>3 years 0 months</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>1.2</v>
+        <v>3</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>high school</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Hifah Technologies | Abbottabad Bachelor of Software Engineering</t>
+          <t>Higher school January 2020– March 2022</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>date_range via fuzzy-month + month-name + year-only</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M22" t="n">
-        <v>63.21</v>
+        <v>63.38</v>
       </c>
       <c r="N22" t="n">
         <v>21</v>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>matplotlib, scikit-learn, python, mysql, hive, statistics, sql, r, github, monitoring, machine learning, communication, aws, spark, ec2, hadoop, git, data visualization, s3, tensorflow, sqlite</t>
+          <t>mysql, ec2, hive, sqlite, data visualization, r, aws, hadoop, github, python, tensorflow, machine learning, git, monitoring, scikit-learn, s3, matplotlib, communication, sql, spark, statistics</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>postgresql, kubernetes, python, mysql, nosql, hive, flask, agile, sql, mongodb, azure, github, monitoring, java, cassandra, machine learning, aws, spark, problem solving, ec2, hadoop, s3, rest api, docker</t>
+          <t>mysql, ec2, hive, kubernetes, aws, flask, hadoop, github, python, java, machine learning, agile, problem solving, nosql, postgresql, azure, mongodb, monitoring, s3, rest api, sql, spark, docker, cassandra</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1963,7 +1963,7 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>postgresql, react.js, figma, python, php, mysql, nosql, agile, sql, firebase, react, node.js, typescript, vite, tailwind css, github, angular, vercel, css, redux, laravel, javascript, project management, flutter, next.js, sass, git, django, mongodb, express</t>
+          <t>mysql, project management, react, typescript, css, figma, github, next.js, python, php, node.js, tailwind css, laravel, agile, react.js, nosql, postgresql, git, mongodb, javascript, django, vite, vercel, sql, firebase, flutter, express, sass, angular, redux</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1990,7 +1990,7 @@
         </is>
       </c>
       <c r="M25" t="n">
-        <v>62.95</v>
+        <v>62.62</v>
       </c>
       <c r="N25" t="n">
         <v>24</v>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>jwt, react.js, python, sql, firebase, react, node.js, r, tailwind css, github, authorization, css, redux, authentication, javascript, flutter, html, state management, git, mongodb, express</t>
+          <t>react, authentication, css, r, jwt, github, python, node.js, tailwind css, react.js, git, mongodb, authorization, html, javascript, sql, firebase, state management, flutter, express, redux</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2056,7 +2056,7 @@
         </is>
       </c>
       <c r="M26" t="n">
-        <v>61.28</v>
+        <v>61.62</v>
       </c>
       <c r="N26" t="n">
         <v>25</v>
@@ -2087,7 +2087,7 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>jenkins, kubernetes, python, bitbucket, mysql, docker, hive, kafka, redshift, sql, azure, github, monitoring, cloudwatch, java, cassandra, authentication, aws, spark, bigquery, hadoop, git, grafana, s3, rest api, linux</t>
+          <t>mysql, jenkins, bitbucket, kafka, hive, authentication, kubernetes, aws, hadoop, github, python, java, azure, git, cloudwatch, monitoring, grafana, s3, rest api, linux, sql, spark, docker, cassandra, bigquery, redshift</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2123,64 +2123,60 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1-Fahadalamresume.pdf</t>
+          <t>Nezuko_Kamado_Resume_10-08-2022-16-04-20.pdf</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Fahad Alam</t>
+          <t>Kamado Associate Lead</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>fahadalam12405@gmail.com</t>
+          <t>hello.ineuron@gmail.com</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>+923272748498</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/fahad-alam</t>
-        </is>
-      </c>
+          <t>9923312341</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://github.com/Fahad12405</t>
+          <t>https://github.com/model</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>vue.js, react.js, firebase, react, node.js, typescript, vite, tailwind css, github, jquery, webpack, context api, css, redux, postcss, javascript, redux toolkit, html, axios, next.js, state management, git, bootstrap, mongodb, express</t>
+          <t>gcp, grpc, kafka, prometheus, keras, kubernetes, aws, flask, seaborn, github, python, numpy, pandas, linear regression, tensorflow, machine learning, azure, pytorch, grafana, deep learning, rest api, matplotlib, django, clustering, fastapi, docker, probability, statistics, dimensionality</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1 years 3 months</t>
+          <t>6 years 0 months</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>high school</t>
+          <t>bachelor</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Intermediate, Cs</t>
+          <t>Bachelor Of Technology in Computer Science</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>date_range via reverse-order</t>
+          <t>summary via summary</t>
         </is>
       </c>
       <c r="M28" t="n">
-        <v>60.19</v>
+        <v>60.08</v>
       </c>
       <c r="N28" t="n">
         <v>27</v>
@@ -2189,60 +2185,64 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Nezuko_Kamado_Resume_10-08-2022-16-04-20.pdf</t>
+          <t>1-Fahadalamresume.pdf</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Kamado Associate Lead</t>
+          <t>Fahad Alam</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>hello.ineuron@gmail.com</t>
+          <t>fahadalam12405@gmail.com</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>9923312341</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
+          <t>+923272748498</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/fahad-alam</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://github.com/model</t>
+          <t>https://github.com/Fahad12405</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>matplotlib, kubernetes, python, flask, statistics, kafka, gcp, linear regression, pandas, deep learning, azure, probability, github, numpy, seaborn, prometheus, clustering, machine learning, dimensionality, aws, grpc, fastapi, django, grafana, tensorflow, pytorch, rest api, keras, docker</t>
+          <t>react, axios, typescript, context api, css, redux toolkit, vue.js, postcss, github, next.js, bootstrap, node.js, tailwind css, react.js, git, mongodb, jquery, webpack, html, javascript, vite, firebase, state management, express, redux</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>6 years 0 months</t>
+          <t>1 years 3 months</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>bachelor</t>
+          <t>high school</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Bachelor Of Technology in Computer Science</t>
+          <t>Intermediate, Cs</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>summary via summary</t>
+          <t>date_range via reverse-order</t>
         </is>
       </c>
       <c r="M29" t="n">
-        <v>60.08</v>
+        <v>59.69</v>
       </c>
       <c r="N29" t="n">
         <v>28</v>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>yarn, html, next.js, react, firebase, react.js, css, redux, git, authentication, react router, github, javascript, redux toolkit, npm, vercel</t>
+          <t>redux, css, react router, react, react.js, firebase, npm, redux toolkit, git, vercel, authentication, yarn, github, next.js, html, javascript</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>html, react, node.js, react.js, figma, typescript, css, bootstrap, netlify, nosql, github, javascript, mongodb, express, sql</t>
+          <t>bootstrap, node.js, css, react, figma, react.js, nosql, sql, mongodb, typescript, express, github, netlify, html, javascript</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>matplotlib, streamlit, python, mysql, load balancing, sql, pandas, github, vs code, numpy, seaborn,  hypothesis testing, css, machine learning, communication, jupyter, javascript, project management, html, critical thinking, git, decision trees, jupyter notebook</t>
+          <t>mysql, project management, jupyter, critical thinking,  hypothesis testing, css, streamlit, seaborn, github, python, numpy, pandas, vs code, machine learning, git, html, javascript, matplotlib, load balancing, decision trees, communication, sql, jupyter notebook</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>matplotlib, streamlit, python, mysql, load balancing, plotly, sql, linear regression, pandas, probability, github, vs code, numpy, seaborn, clustering,  hypothesis testing, css, dimensionality, machine learning, communication, jupyter, cross-validation, javascript, project management, supervised, html, feature engineering, etl pipelines, unsupervised learning, hyperparameter tuning, git, decision trees, jupyter notebook, linux</t>
+          <t>mysql, project management, feature engineering, jupyter, unsupervised learning, etl pipelines, hyperparameter tuning,  hypothesis testing, css, cross-validation, streamlit, seaborn, plotly, github, python, numpy, pandas, vs code, linear regression, machine learning, git, supervised, html, javascript, matplotlib, load balancing, clustering, decision trees, communication, linux, sql, probability, dimensionality, jupyter notebook</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>clustering, deep learning,  hypothesis testing, azure, python, machine learning, probability, kafka, jupyter notebook, jupyter, github, aws, statistics, spark, docker</t>
+          <t>aws, clustering, machine learning, jupyter notebook, jupyter, spark, docker, probability, statistics, kafka, azure,  hypothesis testing, github, python, deep learning</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>responsive design, jwt, react.js, nosql, sql, react hooks, firebase, react, node.js, lazy loading, netlify, tailwind css, github, jquery, java, css, redux, authentication, android, aws, javascript, react native, state management, kotlin, mongodb, express</t>
+          <t>react, authentication, kotlin, css, aws, jwt, github, java, netlify, android, node.js, tailwind css, react.js, nosql, responsive design, mongodb, react native, jquery, javascript, react hooks, firebase, sql, state management, lazy loading, express, redux</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>html, java, react, node.js, react.js, material ui, css, communication, github, mongodb, express</t>
+          <t>node.js, communication, css, react, react.js, material ui, mongodb, github, java, express, html</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2727,7 +2727,7 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>deep learning, azure, python, machine learning, kafka, aws, spark, docker</t>
+          <t>aws, machine learning, azure, spark, docker, kafka, python, deep learning</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2789,7 +2789,7 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>next.js, react, problem solving, react.js, responsive design, css, git, bootstrap, communication, tailwind css, r, javascript</t>
+          <t>bootstrap, tailwind css, communication, react, react.js, problem solving, responsive design, git, r, next.js, css, javascript</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2816,7 +2816,7 @@
         </is>
       </c>
       <c r="M38" t="n">
-        <v>53.96</v>
+        <v>54.46</v>
       </c>
       <c r="N38" t="n">
         <v>37</v>
@@ -2901,7 +2901,7 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>html, .net, css, communication, monitoring, asp.net, agile, javascript, project management, sql</t>
+          <t>project management, communication, agile, css, .net, sql, asp.net, monitoring, html, javascript</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>matplotlib, streamlit, python, mysql, plotly, flask, sql, pandas, deep learning, github, numpy, css, machine learning, aws, html, feature engineering, ec2, express, git, django, redis, mongodb, docker</t>
+          <t>mysql, feature engineering, ec2, css, aws, flask, streamlit, plotly, github, python, numpy, pandas, machine learning, git, mongodb, html, deep learning, matplotlib, django, sql, docker, express, redis</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>axios, react, mongodb, typescript, php, css, redux, mysql, sass, git, tailwind css, github, javascript, jquery, vercel, sql</t>
+          <t>mysql, redux, tailwind css, vercel, react, sql, git, axios, mongodb, typescript, jquery, github, sass, php, css, javascript</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3056,7 +3056,7 @@
         </is>
       </c>
       <c r="M42" t="n">
-        <v>45.71</v>
+        <v>45.54</v>
       </c>
       <c r="N42" t="n">
         <v>41</v>
@@ -3087,7 +3087,7 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>deep learning,  hypothesis testing, azure, python, machine learning, probability, kafka, aws, statistics, spark, docker</t>
+          <t>aws, machine learning, azure, spark, docker, probability, statistics, kafka,  hypothesis testing, python, deep learning</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3149,7 +3149,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>linear regression, problem solving, kubernetes, deep learning, cassandra, python, machine learning, mysql, tensorflow, github, pytorch, aws, mongodb, docker</t>
+          <t>kubernetes, tensorflow, mysql, aws, machine learning, problem solving, cassandra, docker, pytorch, mongodb, github, python, deep learning, linear regression</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -3211,7 +3211,7 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>html, next.js, react, css, bootstrap, github</t>
+          <t>bootstrap, css, react, github, next.js, html</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3269,7 +3269,7 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>prometheus, firewalls, siem, network security, python, machine learning, git, data visualization, gitlab, monitoring, gitlab ci, aws, linux</t>
+          <t>aws, gitlab, machine learning, linux, gitlab ci, siem, firewalls, git, python, prometheus, network security, monitoring, data visualization</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3327,7 +3327,7 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>communication, critical thinking</t>
+          <t>critical thinking, communication</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">

</xml_diff>

<commit_message>
not logging bug fixed
</commit_message>
<xml_diff>
--- a/output/all_candidates_ranked.xlsx
+++ b/output/all_candidates_ranked.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,60 +441,65 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>GitHub</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Skills</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Experience</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Experience (Years)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Raw Education</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Experience Method</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
@@ -513,56 +518,61 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>mominhyatkhandeveloper@gmail.com</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>03345674415</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>https://linkedin.com/in/mominhyatkhan</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>https://github.com/mominhyatkhan</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>mysql, react, axios, authentication, hive, typescript, css, nest.js, integration testing, jwt, eslint, material ui, spring boot, github, next.js, java, react query, redux, tailwind css, agile, git, authorization, spring, monitoring, html, javascript, oauth, prettier, unit testing</t>
-        </is>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>github, integration testing, eslint, redux, hive, next.js, typescript, javascript, mysql, unit testing, oauth, css, prettier, java, react, material ui, jwt, spring boot, axios, agile, react query, monitoring, authentication, git, authorization, html, spring, nest.js, tailwind css</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>4 years 0 months</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>4</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>87.69</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -579,56 +589,61 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>React.Js Developer</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>zeeshanzahoor409@gmail.com</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>+923421905266</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/zeeshan-zahoor-220b0b130</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>https://github.com/zeeshanshaanu</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>react, authentication, typescript, data visualization, css, figma, redux toolkit, material ui, github, lighthouse, next.js, netlify, vs code, bootstrap, node.js, tailwind css, react.js, responsive design, git, mongodb, javascript, communication, vercel, websockets, express, redux</t>
-        </is>
-      </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>github, redux, responsive design, vercel, websockets, next.js, data visualization, react.js, vs code, typescript, figma, javascript, css, mongodb, express, redux toolkit, react, communication, material ui, bootstrap, authentication, git, netlify, tailwind css, node.js, lighthouse</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>3 years 0 months</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>3</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>🎓 BS in Computer Science (2016 – 2020) | Gov’t Post Graduate College, Haripur</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>87.69</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>2</v>
       </c>
     </row>
@@ -645,56 +660,61 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>React.Js Developer</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>zeeshanzahoor409@gmail.com</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>+923421905266</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/zeeshan-zahoor-220b0b130</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>https://github.com/zeeshanshaanu</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>react, authentication, typescript, data visualization, css, figma, redux toolkit, material ui, github, lighthouse, next.js, netlify, vs code, bootstrap, node.js, tailwind css, react.js, responsive design, git, mongodb, javascript, communication, vercel, websockets, express, redux</t>
-        </is>
-      </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>github, redux, responsive design, vercel, websockets, next.js, data visualization, react.js, vs code, typescript, figma, javascript, css, mongodb, express, redux toolkit, react, communication, material ui, bootstrap, authentication, git, netlify, tailwind css, node.js, lighthouse</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>3 years 0 months</t>
         </is>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>3</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>🎓 BS in Computer Science (2016 – 2020) | Gov’t Post Graduate College, Haripur</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>87.69</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -711,56 +731,61 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Stack Developer</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>muhammadfaizanjanjua109@gmail.com</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>+923405966112</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/follow-muhammadfaizan/</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>https://github.com/Muhammadfaizanjanjua109</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>react, graphql, typescript, css, aws, cypress, figma, vue.js, seo optimization, scrum, github, next.js, netlify, node.js, tailwind css, agile, react.js, code splitting, github actions, responsive design, postgresql, styled components, git, mongodb, react testing library, webpack, javascript, jest, vercel, docker, state management, babel, single page applications, lazy loading, progressive web apps, express, redux</t>
-        </is>
-      </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>progressive web apps, github, redux, responsive design, vue.js, vercel, next.js, postgresql, code splitting, babel, react.js, typescript, figma, javascript, css, graphql, mongodb, express, seo optimization, cypress, styled components, react, react testing library, agile, aws, lazy loading, single page applications, docker, git, jest, netlify, scrum, github actions, webpack, tailwind css, state management, node.js</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>3 years 0 months</t>
         </is>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>3</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Bachelor of Science in Software Engineering</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>84.62</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>4</v>
       </c>
     </row>
@@ -777,52 +802,57 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Full-Stack Developer</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>abdullahkh1144@gmail.com</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>+923105778487</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>https://linkedin.com/in/abdullah-khan-0727b0247</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>project management, react, authentication, graphql, typescript, css, aws, seo optimization, next.js, bootstrap, redux, node.js, tailwind css, agile, react.js, azure, responsive design, git, mongodb, javascript, communication, firebase, websockets, unit testing</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
+          <t>project management, redux, firebase, azure, responsive design, websockets, next.js, react.js, typescript, javascript, unit testing, css, graphql, mongodb, seo optimization, react, communication, bootstrap, agile, aws, authentication, git, tailwind css, node.js</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>5 years 0 months</t>
         </is>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>5</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Bachelor of Science in SOFTWARE ENGINEERING</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>82.62</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>5</v>
       </c>
     </row>
@@ -839,56 +869,61 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>pakistan03479@gmail.com</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>+923139131611</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>https://linkedin.com/in/ayazcoder</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>https://github.com/ayazcoder</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>mysql, project management, react, css, material ui, scrum, github, python, android, node.js, tailwind css, react.js, github actions, azure, git, mongodb, javascript, communication, react hooks, ios, firebase, flutter, express</t>
-        </is>
-      </c>
       <c r="H7" t="inlineStr">
         <is>
+          <t>project management, flutter, github, firebase, azure, react.js, javascript, mysql, css, mongodb, express, python, react, communication, ios, material ui, react hooks, android, git, scrum, github actions, tailwind css, node.js</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
           <t>3 years 2 months</t>
         </is>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>3.2</v>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Bachelor of Software Engineering</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>81.54000000000001</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>6</v>
       </c>
     </row>
@@ -905,52 +940,57 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>saqibifitkhar756@gmail.com</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>03403118722</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/saqib--iftikhar</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>mysql, react, authentication, css, r, figma, material ui, node.js, tailwind css, laravel, agile, react.js, git, mongodb, authorization, html, javascript, communication, state management, express, redux</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
+          <t>redux, react.js, figma, javascript, mysql, css, mongodb, express, react, communication, material ui, agile, authentication, git, laravel, r, authorization, html, tailwind css, state management, node.js</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
           <t>2 years 6 months</t>
         </is>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>2.5</v>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>BS (COMPUTER SCIENCE) ( 2018 - 2022 )</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>80.69</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>7</v>
       </c>
     </row>
@@ -967,48 +1007,53 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>junaidjojo4@gmail.com</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>+923337661597</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>bootstrap, tailwind css, react, figma, react.js, linux, git, material ui, typescript, adobe xd, github, next.js, css, javascript</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
+          <t>linux, github, react.js, git, typescript, adobe xd, figma, react, material ui, javascript, bootstrap, tailwind css, next.js, css</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t>3 years 0 months</t>
         </is>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>3</v>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Bachelor of Science in Software Engineering</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>79.62</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1025,56 +1070,61 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>samikhaan7814@gmail.com</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>+923443777814</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>https://linkedin.com/in/sami-khan-111678169</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>https://github.com/mr-samikhan</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>aws, bootstrap, redux, tailwind css, machine learning, vercel, react, firebase, azure, docker, material ui, mongodb, api's integration, github, php, express, css</t>
-        </is>
-      </c>
       <c r="H10" t="inlineStr">
         <is>
+          <t>api's integration, express, github, redux, react, firebase, machine learning, azure, php, material ui, bootstrap, vercel, tailwind css, aws, css, mongodb, docker</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
           <t>3 years 0 months</t>
         </is>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>3</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>BS Computer Science</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>78.45999999999999</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1091,48 +1141,53 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>End Developer</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>mtahayasin07@gmail.com</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>03406991719</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>bootstrap, tailwind css, vite, css, npm, react, figma, react.js, yarn, problem solving, git, chrome devtools, vs code, github, html, javascript</t>
-        </is>
-      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
+          <t>github, react.js, git, vs code, figma, problem solving, react, yarn, chrome devtools, html, javascript, bootstrap, tailwind css, npm, vite, css</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
           <t>5 years 6 months</t>
         </is>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>5.5</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>BS Software Engineering</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>date_range via month-name + year-only + year-only + year-only-fuzzy</t>
         </is>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>76.54000000000001</v>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1149,48 +1204,53 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>Stack Developer</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>rehanansari3973@gmail.com</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>03099332253</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>mysql, project management, react, authentication, typescript, css, ci/cd pipelines, aws, cypress, figma, jwt, redux toolkit, node.js, tailwind css, agile, react.js, responsive design, git, mongodb, teamwork, html, javascript, communication, jest, react hooks, state management, lazy loading, express, redux</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
+          <t>project management, redux, responsive design, react.js, typescript, figma, javascript, mysql, ci/cd pipelines, css, mongodb, express, redux toolkit, cypress, react, communication, jwt, agile, aws, lazy loading, react hooks, teamwork, authentication, git, jest, html, tailwind css, state management, node.js</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
           <t>2 years 4 months</t>
         </is>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>2.3</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>I pursued Bachelor of Science in Computer Science (BSc CS) from GC University.</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
-      <c r="M12" t="n">
+      <c r="N12" t="n">
         <v>75.69</v>
       </c>
-      <c r="N12" t="n">
+      <c r="O12" t="n">
         <v>11</v>
       </c>
     </row>
@@ -1207,48 +1267,53 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>Unity Developer</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t>Mwbkkj@gmail.com</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>03126318724</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>android, redux, project management, css, react, react.js, ios, firebase, state management, github, python, html, javascript</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
+          <t>project management, python, github, android, react.js, redux, react, firebase, ios, html, javascript, state management, css</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
           <t>3 years 0 months</t>
         </is>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
         <v>3</v>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>master</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Master of Management Science (Finance-18 year edu) from IMSciences, Hayatabad</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M13" t="n">
+      <c r="N13" t="n">
         <v>73.45999999999999</v>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1265,48 +1330,53 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>Frontend Engineer</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>ijlalshahzr@gmail.com</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>+923181669799</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>react, authentication, typescript, context api, css, redux toolkit, material ui, bootstrap, agile, react.js, git, mongodb, asp.net, authorization, jquery, monitoring, html, javascript, communication, .net, react hooks, sql, state management, lazy loading, angular, redux</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
+          <t>context api, redux, jquery, react.js, typescript, javascript, css, mongodb, redux toolkit, react, sql, communication, material ui, bootstrap, agile, monitoring, lazy loading, react hooks, authentication, asp.net, git, .net, authorization, html, state management, angular</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
           <t>2 years 0 months</t>
         </is>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
         <v>2</v>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M14" t="n">
+      <c r="N14" t="n">
         <v>72.69</v>
       </c>
-      <c r="N14" t="n">
+      <c r="O14" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1323,56 +1393,61 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>thedev.hamza@gmail.com</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>03168767587</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/hamxa-hamid/</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>https://github.com/dadhsahb</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>gcp, react, css, aws, vue.js, github, java, bootstrap, node.js, tailwind css, react.js, azure, postgresql, git, mongodb, asp.net, jquery, html, s3, javascript, .net, sql, docker, express, chakra ui</t>
-        </is>
-      </c>
       <c r="H15" t="inlineStr">
         <is>
+          <t>github, azure, vue.js, postgresql, jquery, gcp, react.js, javascript, css, mongodb, express, java, sql, react, chakra ui, bootstrap, aws, docker, asp.net, git, .net, s3, html, tailwind css, node.js</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
           <t>1 years 11 months</t>
         </is>
       </c>
-      <c r="I15" t="n">
+      <c r="J15" t="n">
         <v>1.9</v>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>Bachelor of Science</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>date_range via mm/yyyy + year-only</t>
         </is>
       </c>
-      <c r="M15" t="n">
+      <c r="N15" t="n">
         <v>70.54000000000001</v>
       </c>
-      <c r="N15" t="n">
+      <c r="O15" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1389,48 +1464,53 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>lehazalil23@gmail.com</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>03488899315</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>node.js, tailwind css, css, react, react.js, responsive design, material ui, mongodb, typescript, next.js, express, html, javascript</t>
-        </is>
-      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
+          <t>express, react.js, node.js, typescript, react, html, responsive design, javascript, material ui, tailwind css, next.js, css, mongodb</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
           <t>2 years 0 months</t>
         </is>
       </c>
-      <c r="I16" t="n">
+      <c r="J16" t="n">
         <v>2</v>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>BS Software Engineering Jan 2020 - Feb 2024</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M16" t="n">
+      <c r="N16" t="n">
         <v>69.62</v>
       </c>
-      <c r="N16" t="n">
+      <c r="O16" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1447,56 +1527,61 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>chaqib4u@gmail.com</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>+923040505345</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/aqib-zaib-</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>https://github.com/aqibzaib</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>redux, tailwind css, vercel, react, vue.js, figma, react.js, redux toolkit, git, github, next.js, react query, css, javascript</t>
-        </is>
-      </c>
       <c r="H17" t="inlineStr">
         <is>
+          <t>github, react.js, git, figma, redux, redux toolkit, react, javascript, vercel, vue.js, tailwind css, next.js, react query, css</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
           <t>1 years 6 months</t>
         </is>
       </c>
-      <c r="I17" t="n">
+      <c r="J17" t="n">
         <v>1.5</v>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>BS SOFTWARE</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>date_range via mm/yyyy + year-only</t>
         </is>
       </c>
-      <c r="M17" t="n">
+      <c r="N17" t="n">
         <v>66.54000000000001</v>
       </c>
-      <c r="N17" t="n">
+      <c r="O17" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1513,48 +1598,53 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>shubham.mishra@gmail.com</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>9876543210</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>mysql, bitbucket, kafka, hive, kubernetes, aws, flask, hadoop, github, python, java, bootstrap, azure, git, cloudwatch, monitoring, grafana, s3, rest api, javascript, django, linux, sql, spark, docker, cassandra, bigquery, redshift</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
+          <t>django, github, azure, hive, grafana, kubernetes, flask, cloudwatch, bigquery, javascript, mysql, cassandra, linux, python, java, sql, bootstrap, rest api, bitbucket, aws, monitoring, docker, git, redshift, s3, spark, kafka, hadoop</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
           <t>3 years 0 months</t>
         </is>
       </c>
-      <c r="I18" t="n">
+      <c r="J18" t="n">
         <v>3</v>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>master</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>Master of Computer Applications</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M18" t="n">
+      <c r="N18" t="n">
         <v>64.23</v>
       </c>
-      <c r="N18" t="n">
+      <c r="O18" t="n">
         <v>17</v>
       </c>
     </row>
@@ -1571,48 +1661,53 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>rahul.mishra@gmail.com</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>9876543210</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>mysql, bitbucket, kafka, hive, kubernetes, aws, flask, hadoop, github, python, java, bootstrap, azure, git, cloudwatch, monitoring, grafana, s3, rest api, javascript, django, linux, sql, spark, docker, cassandra, bigquery, redshift</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
+          <t>django, github, azure, hive, grafana, kubernetes, flask, cloudwatch, bigquery, javascript, mysql, cassandra, linux, python, java, sql, bootstrap, rest api, bitbucket, aws, monitoring, docker, git, redshift, s3, spark, kafka, hadoop</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
           <t>4 years 0 months</t>
         </is>
       </c>
-      <c r="I19" t="n">
+      <c r="J19" t="n">
         <v>4</v>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>master</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>Master of Computer Applications, National Institute of Technology Allahabad (MNNIT), U.P</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M19" t="n">
+      <c r="N19" t="n">
         <v>64.23</v>
       </c>
-      <c r="N19" t="n">
+      <c r="O19" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1629,56 +1724,61 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>Front-End Developer</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>yasinwaheed11@gmail.com</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>+923026770777</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/yasinwahid111</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>https://github.com/YasinWahid</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>bootstrap, communication, css, react, figma, react.js, firebase, responsive design, git, react native, typescript, github, angular, html, javascript</t>
-        </is>
-      </c>
       <c r="H20" t="inlineStr">
         <is>
+          <t>react native, github, react.js, git, typescript, figma, firebase, react, communication, html, css, responsive design, javascript, bootstrap, angular</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
           <t>1 years 2 months</t>
         </is>
       </c>
-      <c r="I20" t="n">
+      <c r="J20" t="n">
         <v>1.2</v>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>Hifah Technologies | Abbottabad Bachelor of Software Engineering</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>date_range via fuzzy-month + month-name + year-only</t>
         </is>
       </c>
-      <c r="M20" t="n">
+      <c r="N20" t="n">
         <v>63.54</v>
       </c>
-      <c r="N20" t="n">
+      <c r="O20" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1695,52 +1795,57 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>Js Developer</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
           <t>ayanejaz420fwisg_dpy@indeedemail.com</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>+923313322420</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>https://linkedin.com/in/ejaz-ahmad-2359a2247</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>css, react, mongodb, less, graphql, typescript, html, rest api</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
+          <t>typescript, react, html, less, rest api, css, graphql, mongodb</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
           <t>2 years 0 months</t>
         </is>
       </c>
-      <c r="I21" t="n">
+      <c r="J21" t="n">
         <v>2</v>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M21" t="n">
+      <c r="N21" t="n">
         <v>63.38</v>
       </c>
-      <c r="N21" t="n">
+      <c r="O21" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1757,52 +1862,57 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>Stack Developer</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>kshayan091@gmail.com</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>+923168104861</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/shayan-khan20</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>react, authentication, typescript, aws, figma, jwt, material ui, seo optimization, github, rails, next.js, node.js, mongodb, react native, javascript, ruby, oauth, firebase, express, redux</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
+          <t>github, redux, firebase, next.js, react native, ruby, typescript, figma, javascript, oauth, mongodb, express, seo optimization, react, material ui, jwt, aws, authentication, rails, node.js</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
           <t>3 years 0 months</t>
         </is>
       </c>
-      <c r="I22" t="n">
+      <c r="J22" t="n">
         <v>3</v>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>high school</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>Higher school January 2020– March 2022</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M22" t="n">
+      <c r="N22" t="n">
         <v>63.38</v>
       </c>
-      <c r="N22" t="n">
+      <c r="O22" t="n">
         <v>21</v>
       </c>
     </row>
@@ -1819,56 +1929,61 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>Data Scientist</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
           <t>juanjose.carin@gmail.com</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>940416503364590</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>https://linkedin.com/in/juanjosecarin</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>https://github.com/juanjocarin/W261-Machine-Learning-At-Scale/blob/master/Week07-MrJob/MIDS-W261-2015-HWK-Week07-CarinLlopSatpati-groupZ.ipynb</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>mysql, ec2, hive, sqlite, data visualization, r, aws, hadoop, github, python, tensorflow, machine learning, git, monitoring, scikit-learn, s3, matplotlib, communication, sql, spark, statistics</t>
-        </is>
-      </c>
       <c r="H23" t="inlineStr">
         <is>
+          <t>github, tensorflow, hive, data visualization, mysql, scikit-learn, matplotlib, python, sql, machine learning, communication, ec2, monitoring, aws, git, r, spark, s3, hadoop, sqlite, statistics</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
           <t>5 years 1 months</t>
         </is>
       </c>
-      <c r="I23" t="n">
+      <c r="J23" t="n">
         <v>5.1</v>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>master</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>Master of Information and Data Science</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>date_range via fuzzy-month + month-name + year-only + year-only-fuzzy</t>
         </is>
       </c>
-      <c r="M23" t="n">
+      <c r="N23" t="n">
         <v>63.08</v>
       </c>
-      <c r="N23" t="n">
+      <c r="O23" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1885,56 +2000,61 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
           <t>bisjwa1445@gmail.com</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>+91987654321</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/11i/</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>https://github.com/AnkitDB9</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>mysql, ec2, hive, kubernetes, aws, flask, hadoop, github, python, java, machine learning, agile, problem solving, nosql, postgresql, azure, mongodb, monitoring, s3, rest api, sql, spark, docker, cassandra</t>
-        </is>
-      </c>
       <c r="H24" t="inlineStr">
         <is>
+          <t>github, azure, hive, kubernetes, postgresql, flask, problem solving, mysql, mongodb, cassandra, python, java, sql, machine learning, nosql, rest api, agile, ec2, aws, monitoring, docker, spark, s3, hadoop</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
           <t>4 years 8 months</t>
         </is>
       </c>
-      <c r="I24" t="n">
+      <c r="J24" t="n">
         <v>4.7</v>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>Bachelor of Technology,</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>date_range via fuzzy-month + month-name + year-only + year-only-fuzzy</t>
         </is>
       </c>
-      <c r="M24" t="n">
+      <c r="N24" t="n">
         <v>63.08</v>
       </c>
-      <c r="N24" t="n">
+      <c r="O24" t="n">
         <v>23</v>
       </c>
     </row>
@@ -1951,48 +2071,53 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
           <t>tayabsajid5@gmail.com</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>+923365298230</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>mysql, project management, react, typescript, css, figma, github, next.js, python, php, node.js, tailwind css, laravel, agile, react.js, nosql, postgresql, git, mongodb, javascript, django, vite, vercel, sql, firebase, flutter, express, sass, angular, redux</t>
-        </is>
-      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
+          <t>project management, flutter, django, github, redux, firebase, vercel, next.js, postgresql, react.js, typescript, figma, javascript, mysql, vite, css, mongodb, express, python, sql, react, nosql, agile, sass, git, laravel, php, tailwind css, angular, node.js</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
           <t>1 years 4 months</t>
         </is>
       </c>
-      <c r="I25" t="n">
+      <c r="J25" t="n">
         <v>1.3</v>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>Bachelor of Science in Software Engineering</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
-      <c r="M25" t="n">
+      <c r="N25" t="n">
         <v>62.62</v>
       </c>
-      <c r="N25" t="n">
+      <c r="O25" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2009,56 +2134,61 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
           <t>saadahmad6830879@gmail.com</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>923176830879</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>https://linkedin.com/in/saadahmad879</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>https://github.com/SaADii09</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>react, authentication, css, r, jwt, github, python, node.js, tailwind css, react.js, git, mongodb, authorization, html, javascript, sql, firebase, state management, flutter, express, redux</t>
-        </is>
-      </c>
       <c r="H26" t="inlineStr">
         <is>
+          <t>flutter, github, redux, firebase, react.js, javascript, css, mongodb, express, python, sql, react, jwt, authentication, git, r, authorization, html, tailwind css, state management, node.js</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
           <t>0 years 8 months</t>
         </is>
       </c>
-      <c r="I26" t="n">
+      <c r="J26" t="n">
         <v>0.7</v>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>BS Computer Science</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
-      <c r="M26" t="n">
+      <c r="N26" t="n">
         <v>61.62</v>
       </c>
-      <c r="N26" t="n">
+      <c r="O26" t="n">
         <v>25</v>
       </c>
     </row>
@@ -2075,48 +2205,53 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
           <t>shubham.mishra@gmail.com</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>9876543210</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>mysql, jenkins, bitbucket, kafka, hive, authentication, kubernetes, aws, hadoop, github, python, java, azure, git, cloudwatch, monitoring, grafana, s3, rest api, linux, sql, spark, docker, cassandra, bigquery, redshift</t>
-        </is>
-      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
+          <t>github, azure, hive, grafana, kubernetes, cloudwatch, bigquery, mysql, cassandra, jenkins, linux, python, java, sql, rest api, bitbucket, aws, monitoring, docker, authentication, git, redshift, s3, spark, kafka, hadoop</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
           <t>7 years 0 months</t>
         </is>
       </c>
-      <c r="I27" t="n">
+      <c r="J27" t="n">
         <v>7</v>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>Bachelor of Engineering in Computer Science,</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M27" t="n">
+      <c r="N27" t="n">
         <v>61.15</v>
       </c>
-      <c r="N27" t="n">
+      <c r="O27" t="n">
         <v>26</v>
       </c>
     </row>
@@ -2133,52 +2268,57 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
+          <t>Associate Lead</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
           <t>hello.ineuron@gmail.com</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>9923312341</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr">
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
         <is>
           <t>https://github.com/model</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>gcp, grpc, kafka, prometheus, keras, kubernetes, aws, flask, seaborn, github, python, numpy, pandas, linear regression, tensorflow, machine learning, azure, pytorch, grafana, deep learning, rest api, matplotlib, django, clustering, fastapi, docker, probability, statistics, dimensionality</t>
-        </is>
-      </c>
       <c r="H28" t="inlineStr">
         <is>
+          <t>pytorch, probability, deep learning, tensorflow, django, github, azure, grafana, kubernetes, flask, gcp, clustering, fastapi, seaborn, dimensionality, matplotlib, python, numpy, grpc, keras, machine learning, rest api, aws, docker, pandas, linear regression, prometheus, kafka, statistics</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
           <t>6 years 0 months</t>
         </is>
       </c>
-      <c r="I28" t="n">
+      <c r="J28" t="n">
         <v>6</v>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>Bachelor Of Technology in Computer Science</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M28" t="n">
+      <c r="N28" t="n">
         <v>60.08</v>
       </c>
-      <c r="N28" t="n">
+      <c r="O28" t="n">
         <v>27</v>
       </c>
     </row>
@@ -2195,56 +2335,61 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
+          <t>Front-End Developer</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
           <t>fahadalam12405@gmail.com</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>+923272748498</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/fahad-alam</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>https://github.com/Fahad12405</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>react, axios, typescript, context api, css, redux toolkit, vue.js, postcss, github, next.js, bootstrap, node.js, tailwind css, react.js, git, mongodb, jquery, webpack, html, javascript, vite, firebase, state management, express, redux</t>
-        </is>
-      </c>
       <c r="H29" t="inlineStr">
         <is>
+          <t>github, context api, redux, firebase, vue.js, next.js, jquery, react.js, typescript, javascript, vite, css, mongodb, postcss, express, redux toolkit, react, bootstrap, axios, git, html, webpack, tailwind css, state management, node.js</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
           <t>1 years 3 months</t>
         </is>
       </c>
-      <c r="I29" t="n">
+      <c r="J29" t="n">
         <v>1.2</v>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>high school</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>Intermediate, Cs</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>date_range via reverse-order</t>
         </is>
       </c>
-      <c r="M29" t="n">
+      <c r="N29" t="n">
         <v>59.69</v>
       </c>
-      <c r="N29" t="n">
+      <c r="O29" t="n">
         <v>28</v>
       </c>
     </row>
@@ -2261,56 +2406,61 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>Front-End Developer</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
           <t>touseefabid737@gmail.com</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>+923102939875</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/touseefabid</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>https://github.com/Touseef4705</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>redux, css, react router, react, react.js, firebase, npm, redux toolkit, git, vercel, authentication, yarn, github, next.js, html, javascript</t>
-        </is>
-      </c>
       <c r="H30" t="inlineStr">
         <is>
+          <t>authentication, github, react.js, git, redux, redux toolkit, react, firebase, yarn, html, javascript, vercel, react router, npm, next.js, css</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
           <t>1 years 6 months</t>
         </is>
       </c>
-      <c r="I30" t="n">
+      <c r="J30" t="n">
         <v>1.5</v>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>high school</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>Intermediate, Business Commerce</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
-      <c r="M30" t="n">
+      <c r="N30" t="n">
         <v>59.62</v>
       </c>
-      <c r="N30" t="n">
+      <c r="O30" t="n">
         <v>29</v>
       </c>
     </row>
@@ -2327,56 +2477,61 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
+          <t>Js Developer</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
           <t>IK3281751@gmail.com</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>+923361935561</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>https://linkedin.com/in/muhammad-luqman-khan-051047267</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>https://github.com/Luqmanoffical</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>bootstrap, node.js, css, react, figma, react.js, nosql, sql, mongodb, typescript, express, github, netlify, html, javascript</t>
-        </is>
-      </c>
       <c r="H31" t="inlineStr">
         <is>
+          <t>express, github, react.js, node.js, typescript, figma, sql, react, html, netlify, nosql, javascript, bootstrap, css, mongodb</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
           <t>1 years 0 months</t>
         </is>
       </c>
-      <c r="I31" t="n">
+      <c r="J31" t="n">
         <v>1</v>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>Bachelor's Degree in Information Technology</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>date_range via year-only + year-only-fuzzy</t>
         </is>
       </c>
-      <c r="M31" t="n">
+      <c r="N31" t="n">
         <v>58.46</v>
       </c>
-      <c r="N31" t="n">
+      <c r="O31" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2393,56 +2548,61 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
+          <t>Database Administrator</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
           <t>maqeelcs09@gmail.com</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>+923419905547</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>https://linkedin.com/in/aqeelkhan09</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>https://github.com/maqeel019</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>mysql, project management, jupyter, critical thinking,  hypothesis testing, css, streamlit, seaborn, github, python, numpy, pandas, vs code, machine learning, git, html, javascript, matplotlib, load balancing, decision trees, communication, sql, jupyter notebook</t>
-        </is>
-      </c>
       <c r="H32" t="inlineStr">
         <is>
+          <t>project management, github, load balancing, critical thinking, jupyter notebook, vs code, javascript, mysql, seaborn, css,  hypothesis testing, matplotlib, python, numpy, streamlit, sql, machine learning, communication, decision trees, git, jupyter, pandas, html</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
           <t>1 years 6 months</t>
         </is>
       </c>
-      <c r="I32" t="n">
+      <c r="J32" t="n">
         <v>1.5</v>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>Bachelor of Computer Science</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
-      <c r="M32" t="n">
+      <c r="N32" t="n">
         <v>57.31</v>
       </c>
-      <c r="N32" t="n">
+      <c r="O32" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2459,56 +2619,61 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
+          <t>Database Administrator</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
           <t>maqeelcs09@gmail.com</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>+923419905547</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>https://linkedin.com/in/aqeelkhan09</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>https://github.com/maqeel019</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>mysql, project management, feature engineering, jupyter, unsupervised learning, etl pipelines, hyperparameter tuning,  hypothesis testing, css, cross-validation, streamlit, seaborn, plotly, github, python, numpy, pandas, vs code, linear regression, machine learning, git, supervised, html, javascript, matplotlib, load balancing, clustering, decision trees, communication, linux, sql, probability, dimensionality, jupyter notebook</t>
-        </is>
-      </c>
       <c r="H33" t="inlineStr">
         <is>
+          <t>project management, probability, github, load balancing, jupyter notebook, plotly, etl pipelines, unsupervised learning, vs code, clustering, javascript, mysql, hyperparameter tuning, seaborn, css,  hypothesis testing, dimensionality, linux, supervised, matplotlib, python, numpy, streamlit, sql, machine learning, communication, feature engineering, decision trees, git, jupyter, pandas, linear regression, html, cross-validation</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
           <t>1 years 6 months</t>
         </is>
       </c>
-      <c r="I33" t="n">
+      <c r="J33" t="n">
         <v>1.5</v>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>Bachelor of Computer Science</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>date_range via fuzzy-month + month-name + year-only + year-only</t>
         </is>
       </c>
-      <c r="M33" t="n">
+      <c r="N33" t="n">
         <v>57.31</v>
       </c>
-      <c r="N33" t="n">
+      <c r="O33" t="n">
         <v>32</v>
       </c>
     </row>
@@ -2525,52 +2690,57 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
+          <t>Data Scientist</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
           <t>hello.ineuron@gmail.com</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>9923312341</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr">
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
         <is>
           <t>https://github.com/PROFILE</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>aws, clustering, machine learning, jupyter notebook, jupyter, spark, docker, probability, statistics, kafka, azure,  hypothesis testing, github, python, deep learning</t>
-        </is>
-      </c>
       <c r="H34" t="inlineStr">
         <is>
+          <t>kafka, probability, github, deep learning, python, jupyter, clustering, azure, jupyter notebook, machine learning, spark, aws, statistics,  hypothesis testing, docker</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
           <t>4 years 0 months</t>
         </is>
       </c>
-      <c r="I34" t="n">
+      <c r="J34" t="n">
         <v>4</v>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>Bachelor Of Technology in Computer Science, Jaypee Institute Of Information Technology</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M34" t="n">
+      <c r="N34" t="n">
         <v>57</v>
       </c>
-      <c r="N34" t="n">
+      <c r="O34" t="n">
         <v>33</v>
       </c>
     </row>
@@ -2587,52 +2757,57 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
           <t>abdullah.javed9438@gmail.com</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>+923499377144</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr">
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
         <is>
           <t>https://github.com/AbdullahKhanSwati</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>react, authentication, kotlin, css, aws, jwt, github, java, netlify, android, node.js, tailwind css, react.js, nosql, responsive design, mongodb, react native, jquery, javascript, react hooks, firebase, sql, state management, lazy loading, express, redux</t>
-        </is>
-      </c>
       <c r="H35" t="inlineStr">
         <is>
+          <t>github, redux, firebase, responsive design, jquery, react native, react.js, javascript, css, kotlin, mongodb, express, java, sql, react, nosql, jwt, aws, lazy loading, react hooks, authentication, android, netlify, tailwind css, state management, node.js</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
           <t>1 years 0 months</t>
         </is>
       </c>
-      <c r="I35" t="n">
+      <c r="J35" t="n">
         <v>1</v>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>date_range via year-only-fuzzy</t>
         </is>
       </c>
-      <c r="M35" t="n">
+      <c r="N35" t="n">
         <v>55.46</v>
       </c>
-      <c r="N35" t="n">
+      <c r="O35" t="n">
         <v>34</v>
       </c>
     </row>
@@ -2649,56 +2824,61 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
+          <t>Stack Developer</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
           <t>ibrahimahmed12333@gmail.com</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>+923431938944</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/ibrahim-ahmed-8b8961254</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>https://github.com/IbrahimAhmed413</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>node.js, communication, css, react, react.js, material ui, mongodb, github, java, express, html</t>
-        </is>
-      </c>
       <c r="H36" t="inlineStr">
         <is>
+          <t>express, github, react.js, java, node.js, react, communication, html, material ui, css, mongodb</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
           <t>1 years 0 months</t>
         </is>
       </c>
-      <c r="I36" t="n">
+      <c r="J36" t="n">
         <v>1</v>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>Bachelor of Computer Science</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="M36" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M36" t="n">
+      <c r="N36" t="n">
         <v>55.38</v>
       </c>
-      <c r="N36" t="n">
+      <c r="O36" t="n">
         <v>35</v>
       </c>
     </row>
@@ -2715,48 +2895,53 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
+          <t>Data Scientist</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
           <t>Tanjiro.bhatia67@gmail.com</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>9923312341</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>aws, machine learning, azure, spark, docker, kafka, python, deep learning</t>
-        </is>
-      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
+          <t>kafka, python, deep learning, azure, machine learning, spark, aws, docker</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
           <t>6 years 0 months</t>
         </is>
       </c>
-      <c r="I37" t="n">
+      <c r="J37" t="n">
         <v>6</v>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M37" t="n">
+      <c r="N37" t="n">
         <v>55</v>
       </c>
-      <c r="N37" t="n">
+      <c r="O37" t="n">
         <v>36</v>
       </c>
     </row>
@@ -2773,52 +2958,57 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
+          <t>Web Developer</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
           <t>rehmanzeb2k17@gmail.com</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>+923119449029</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/rehmanzeb</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>bootstrap, tailwind css, communication, react, react.js, problem solving, responsive design, git, r, next.js, css, javascript</t>
-        </is>
-      </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
+          <t>react.js, git, problem solving, react, r, communication, responsive design, javascript, bootstrap, tailwind css, next.js, css</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
           <t>0 years 9 months</t>
         </is>
       </c>
-      <c r="I38" t="n">
+      <c r="J38" t="n">
         <v>0.8</v>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>BS Computer Science</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="M38" t="inlineStr">
         <is>
           <t>date_range via fuzzy-month + month-name + year-only + month-only + year</t>
         </is>
       </c>
-      <c r="M38" t="n">
+      <c r="N38" t="n">
         <v>54.46</v>
       </c>
-      <c r="N38" t="n">
+      <c r="O38" t="n">
         <v>37</v>
       </c>
     </row>
@@ -2833,46 +3023,51 @@
           <t>Robin Doe</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr">
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Data Scientist</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
         <is>
           <t>123451234567090</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr">
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
         <is>
           <t>machine learning</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>8 years 6 months</t>
         </is>
       </c>
-      <c r="I39" t="n">
+      <c r="J39" t="n">
         <v>8.5</v>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>ba Eng al) - AMT</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>date_range via year-only + year-only-fuzzy</t>
         </is>
       </c>
-      <c r="M39" t="n">
+      <c r="N39" t="n">
         <v>52</v>
       </c>
-      <c r="N39" t="n">
+      <c r="O39" t="n">
         <v>38</v>
       </c>
     </row>
@@ -2889,48 +3084,53 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
+          <t>Computer Scientist</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
           <t>rabdullah806@gmail.com</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>923175510676</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>project management, communication, agile, css, .net, sql, asp.net, monitoring, html, javascript</t>
-        </is>
-      </c>
+      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
+          <t>project management, asp.net, sql, .net, communication, html, javascript, agile, monitoring, css</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
           <t>1 years 6 months</t>
         </is>
       </c>
-      <c r="I40" t="n">
+      <c r="J40" t="n">
         <v>1.5</v>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>Bachelor (inferred) / No major degree found but mentions university</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="M40" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M40" t="n">
+      <c r="N40" t="n">
         <v>49.23</v>
       </c>
-      <c r="N40" t="n">
+      <c r="O40" t="n">
         <v>39</v>
       </c>
     </row>
@@ -2947,52 +3147,57 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
+          <t>Data Scientist</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
           <t>xyz@gmail.com</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>9977141714</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr">
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
         <is>
           <t>https://github.com/vishalsingh17</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>mysql, feature engineering, ec2, css, aws, flask, streamlit, plotly, github, python, numpy, pandas, machine learning, git, mongodb, html, deep learning, matplotlib, django, sql, docker, express, redis</t>
-        </is>
-      </c>
       <c r="H41" t="inlineStr">
         <is>
+          <t>deep learning, django, github, plotly, redis, flask, mysql, css, mongodb, express, matplotlib, python, numpy, streamlit, sql, machine learning, ec2, aws, docker, feature engineering, git, pandas, html</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
           <t>1 years 0 months</t>
         </is>
       </c>
-      <c r="I41" t="n">
+      <c r="J41" t="n">
         <v>1</v>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>12/2015 – 12/2018 BCA</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="M41" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M41" t="n">
+      <c r="N41" t="n">
         <v>46.23</v>
       </c>
-      <c r="N41" t="n">
+      <c r="O41" t="n">
         <v>40</v>
       </c>
     </row>
@@ -3009,56 +3214,61 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
+          <t>Javascript Developer</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
           <t>jawadalikhan359@gmail.com</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>03139908709</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/jawadali1535</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>https://github.com/JawadAli1535</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>mysql, redux, tailwind css, vercel, react, sql, git, axios, mongodb, typescript, jquery, github, sass, php, css, javascript</t>
-        </is>
-      </c>
       <c r="H42" t="inlineStr">
         <is>
+          <t>jquery, github, tailwind css, git, sass, typescript, redux, react, sql, php, javascript, mysql, vercel, axios, css, mongodb</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
           <t>0 years 5 months</t>
         </is>
       </c>
-      <c r="I42" t="n">
+      <c r="J42" t="n">
         <v>0.4</v>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>high school</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>Nodejs(intermediate)</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="M42" t="inlineStr">
         <is>
           <t>date_range via fuzzy-month + month-name + year-only</t>
         </is>
       </c>
-      <c r="M42" t="n">
+      <c r="N42" t="n">
         <v>45.54</v>
       </c>
-      <c r="N42" t="n">
+      <c r="O42" t="n">
         <v>41</v>
       </c>
     </row>
@@ -3075,48 +3285,53 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
+          <t>Data Scientist</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
           <t>riya.bhatia67@gmail.com</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>9923312341</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>aws, machine learning, azure, spark, docker, probability, statistics, kafka,  hypothesis testing, python, deep learning</t>
-        </is>
-      </c>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
+          <t>kafka, probability, deep learning, python, azure, machine learning, spark, aws, statistics,  hypothesis testing, docker</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
           <t>2 years 0 months</t>
         </is>
       </c>
-      <c r="I43" t="n">
+      <c r="J43" t="n">
         <v>2</v>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>Bachelor Of Technology in Computer Science Freelance Mentor Of Data Structure and Algorithms</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
       </c>
-      <c r="M43" t="n">
+      <c r="N43" t="n">
         <v>45</v>
       </c>
-      <c r="N43" t="n">
+      <c r="O43" t="n">
         <v>42</v>
       </c>
     </row>
@@ -3133,54 +3348,59 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
+          <t>Data Scientist</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
           <t>shankar.chavan@gmail.com</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr">
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
         <is>
           <t>https://in.linkedin.com/</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>https://github.com/</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>kubernetes, tensorflow, mysql, aws, machine learning, problem solving, cassandra, docker, pytorch, mongodb, github, python, deep learning, linear regression</t>
-        </is>
-      </c>
       <c r="H44" t="inlineStr">
         <is>
+          <t>cassandra, pytorch, python, deep learning, tensorflow, github, problem solving, linear regression, machine learning, mysql, kubernetes, aws, mongodb, docker</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
           <t>1 years 6 months</t>
         </is>
       </c>
-      <c r="I44" t="n">
+      <c r="J44" t="n">
         <v>1.5</v>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>master</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>Master Degree, SPPU University</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="M44" t="inlineStr">
         <is>
           <t>summary via summary</t>
         </is>
-      </c>
-      <c r="M44" t="n">
-        <v>43</v>
       </c>
       <c r="N44" t="n">
         <v>43</v>
       </c>
+      <c r="O44" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3195,52 +3415,57 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
+          <t>Software Developer</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
           <t>berlanjan123@gmail.com</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>+923169769253</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/sameer-khan-660966251</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>bootstrap, css, react, github, next.js, html</t>
-        </is>
-      </c>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
+          <t>github, react, html, bootstrap, next.js, css</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
           <t>0 years 0 months</t>
         </is>
       </c>
-      <c r="I45" t="n">
+      <c r="J45" t="n">
         <v>0</v>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>Degree Bs Computer Science</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="M45" t="inlineStr">
         <is>
           <t>none via none</t>
         </is>
       </c>
-      <c r="M45" t="n">
+      <c r="N45" t="n">
         <v>37.23</v>
       </c>
-      <c r="N45" t="n">
+      <c r="O45" t="n">
         <v>44</v>
       </c>
     </row>
@@ -3257,48 +3482,53 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
+          <t>Zeeshan Assistant</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
           <t>muhammadawaisturk1@gmail.com</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>+923155406093</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>aws, gitlab, machine learning, linux, gitlab ci, siem, firewalls, git, python, prometheus, network security, monitoring, data visualization</t>
-        </is>
-      </c>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
+          <t>monitoring, linux, python, gitlab, git, machine learning, siem, network security, gitlab ci, prometheus, aws, firewalls, data visualization</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
           <t>0 years 0 months</t>
         </is>
       </c>
-      <c r="I46" t="n">
+      <c r="J46" t="n">
         <v>0</v>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="L46" t="inlineStr">
         <is>
           <t>BS COMPUTER SCIENCE Abbottabad University Of Science And Technology</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="M46" t="inlineStr">
         <is>
           <t>none via none</t>
         </is>
       </c>
-      <c r="M46" t="n">
+      <c r="N46" t="n">
         <v>28.08</v>
       </c>
-      <c r="N46" t="n">
+      <c r="O46" t="n">
         <v>45</v>
       </c>
     </row>
@@ -3315,48 +3545,53 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
+          <t>To Lead</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
           <t>maqeelcs09@gmail.com</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>+923419905547</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr">
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
         <is>
           <t>critical thinking, communication</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>0 years 0 months</t>
         </is>
       </c>
-      <c r="I47" t="n">
+      <c r="J47" t="n">
         <v>0</v>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>bachelor</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="L47" t="inlineStr">
         <is>
           <t>muhammad abu aqeel nationality: pakistani gender: male phone number: (+92) 3419905547 (mobile) email address: maqeelcs09@gmail.com address: pakistan (home) about me a dedicated individual with a proven track record of achieving and exceeding goals through unwavering determination and a commitment to excellence education and training lahore, pakistan bachelor of science university of swabi field of studycomputer science 2020 bam khel,swabi, pakistan intermediate the glorious college of science &amp; technology language skills mother tongue(s): urdu | pashto other language(s): understanding speaking writing spoken spoken listening reading production interaction english c1 c1 c1 c1 c1 levels: a1 and a2: basic user; b1 and b2: independent user; c1 and c2: proficient user additional information management and leadership skills skills strategic planning and execution: • proficient in developing long-term strategies and effectively executing action plans to achieve organizational goals. • skilled at aligning business objectives with actionable plans for efficient resource utilization. team leadership and motivation: • proven ability to lead and inspire teams, fostering a collaborative and high-performing work environment. • experienced in setting clear expectations, providing constructive feedback, and empowering team members to reach their potential. decision making and problem-solving: • strong analytical and critical thinking skills, enabling effective decision-making in complex situations.</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
+      <c r="M47" t="inlineStr">
         <is>
           <t>none via none</t>
         </is>
       </c>
-      <c r="M47" t="n">
+      <c r="N47" t="n">
         <v>25</v>
       </c>
-      <c r="N47" t="n">
+      <c r="O47" t="n">
         <v>46</v>
       </c>
     </row>

</xml_diff>